<commit_message>
Update Privacy News Dashboard snapshot (2026-09-16 12:20:02 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -1649,7 +1649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1707,17 +1707,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>17151</t>
+          <t>31091</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>개인정보보호위원회 직제 시행규칙 일부개정령안 입법예고</t>
+          <t>개인정보 보호법 시행령 일부개정령안 입법예고</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/lawinfo/makingInfo.mo?mid=a10104010000&amp;lawSeq=88084&amp;lawCd=0&amp;lawType=TYPE5&amp;pageCnt=10&amp;currentPage=1&amp;keyField=lmNm&amp;keyWord=&amp;stYdFmt=&amp;edYdFmt=&amp;lsClsCd=&amp;cptOfiOrgCd=%EA%B0%9C%EC%9D%B8%EC%A0%95%EB%B3%B4%EB%B3%B4%ED%98%B8%EC%9C%84%EC%9B%90%ED%9A%8C</t>
+          <t>https://www.moleg.go.kr/lawinfo/makingInfo.mo?mid=a10104010000&amp;lawSeq=88642&amp;lawCd=0&amp;lawType=TYPE5&amp;pageCnt=10&amp;currentPage=1&amp;keyField=lmNm&amp;keyWord=&amp;stYdFmt=&amp;edYdFmt=&amp;lsClsCd=&amp;cptOfiOrgCd=%EA%B0%9C%EC%9D%B8%EC%A0%95%EB%B3%B4%EB%B3%B4%ED%98%B8%EC%9C%84%EC%9B%90%ED%9A%8C</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1727,49 +1727,49 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>총리령</t>
+          <t>대통령령</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026.08.13</t>
+          <t>2026.09.16</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026.08.20</t>
+          <t>2026.10.26</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-08-13 12:15:11.945277+09:00</t>
+          <t>2026-09-16 12:15:11.569170+09:00</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-08-13 12:15:11.945277+09:00</t>
+          <t>2026-09-16 12:15:11.569170+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>17151</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>개인정보 보호법 시행령 일부개정령안 입법예고</t>
+          <t>개인정보보호위원회 직제 시행규칙 일부개정령안 입법예고</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/lawinfo/makingInfo.mo?mid=a10104010000&amp;lawSeq=87372&amp;lawCd=0&amp;lawType=TYPE5&amp;pageCnt=10&amp;currentPage=1&amp;keyField=lmNm&amp;keyWord=&amp;stYdFmt=&amp;edYdFmt=&amp;lsClsCd=&amp;cptOfiOrgCd=%EA%B0%9C%EC%9D%B8%EC%A0%95%EB%B3%B4%EB%B3%B4%ED%98%B8%EC%9C%84%EC%9B%90%ED%9A%8C</t>
+          <t>https://www.moleg.go.kr/lawinfo/makingInfo.mo?mid=a10104010000&amp;lawSeq=88084&amp;lawCd=0&amp;lawType=TYPE5&amp;pageCnt=10&amp;currentPage=1&amp;keyField=lmNm&amp;keyWord=&amp;stYdFmt=&amp;edYdFmt=&amp;lsClsCd=&amp;cptOfiOrgCd=%EA%B0%9C%EC%9D%B8%EC%A0%95%EB%B3%B4%EB%B3%B4%ED%98%B8%EC%9C%84%EC%9B%90%ED%9A%8C</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1779,39 +1779,39 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>대통령령</t>
+          <t>총리령</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026.06.30</t>
+          <t>2026.08.13</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026.08.10</t>
+          <t>2026.08.20</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:16.444527+09:00</t>
+          <t>2026-08-13 12:15:11.945277+09:00</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:16.444527+09:00</t>
+          <t>2026-08-13 12:15:11.945277+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1821,7 +1821,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/lawinfo/makingInfo.mo?mid=a10104010000&amp;lawSeq=86980&amp;lawCd=0&amp;lawType=TYPE5&amp;pageCnt=10&amp;currentPage=1&amp;keyField=lmNm&amp;keyWord=&amp;stYdFmt=&amp;edYdFmt=&amp;lsClsCd=&amp;cptOfiOrgCd=%EA%B0%9C%EC%9D%B8%EC%A0%95%EB%B3%B4%EB%B3%B4%ED%98%B8%EC%9C%84%EC%9B%90%ED%9A%8C</t>
+          <t>https://www.moleg.go.kr/lawinfo/makingInfo.mo?mid=a10104010000&amp;lawSeq=87372&amp;lawCd=0&amp;lawType=TYPE5&amp;pageCnt=10&amp;currentPage=1&amp;keyField=lmNm&amp;keyWord=&amp;stYdFmt=&amp;edYdFmt=&amp;lsClsCd=&amp;cptOfiOrgCd=%EA%B0%9C%EC%9D%B8%EC%A0%95%EB%B3%B4%EB%B3%B4%ED%98%B8%EC%9C%84%EC%9B%90%ED%9A%8C</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1836,17 +1836,17 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026.06.02</t>
+          <t>2026.06.30</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026.07.13</t>
+          <t>2026.08.10</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1863,7 +1863,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1873,7 +1873,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/lawinfo/makingInfo.mo?mid=a10104010000&amp;lawSeq=86932&amp;lawCd=0&amp;lawType=TYPE5&amp;pageCnt=10&amp;currentPage=1&amp;keyField=lmNm&amp;keyWord=&amp;stYdFmt=&amp;edYdFmt=&amp;lsClsCd=&amp;cptOfiOrgCd=%EA%B0%9C%EC%9D%B8%EC%A0%95%EB%B3%B4%EB%B3%B4%ED%98%B8%EC%9C%84%EC%9B%90%ED%9A%8C</t>
+          <t>https://www.moleg.go.kr/lawinfo/makingInfo.mo?mid=a10104010000&amp;lawSeq=86980&amp;lawCd=0&amp;lawType=TYPE5&amp;pageCnt=10&amp;currentPage=1&amp;keyField=lmNm&amp;keyWord=&amp;stYdFmt=&amp;edYdFmt=&amp;lsClsCd=&amp;cptOfiOrgCd=%EA%B0%9C%EC%9D%B8%EC%A0%95%EB%B3%B4%EB%B3%B4%ED%98%B8%EC%9C%84%EC%9B%90%ED%9A%8C</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1888,7 +1888,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026.06.01</t>
+          <t>2026.06.02</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1898,7 +1898,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1915,17 +1915,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>개인정보보호위원회 직제 시행규칙 일부개정령안 입법예고</t>
+          <t>개인정보 보호법 시행령 일부개정령안 입법예고</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/lawinfo/makingInfo.mo?mid=a10104010000&amp;lawSeq=86700&amp;lawCd=0&amp;lawType=TYPE5&amp;pageCnt=10&amp;currentPage=1&amp;keyField=lmNm&amp;keyWord=&amp;stYdFmt=&amp;edYdFmt=&amp;lsClsCd=&amp;cptOfiOrgCd=%EA%B0%9C%EC%9D%B8%EC%A0%95%EB%B3%B4%EB%B3%B4%ED%98%B8%EC%9C%84%EC%9B%90%ED%9A%8C</t>
+          <t>https://www.moleg.go.kr/lawinfo/makingInfo.mo?mid=a10104010000&amp;lawSeq=86932&amp;lawCd=0&amp;lawType=TYPE5&amp;pageCnt=10&amp;currentPage=1&amp;keyField=lmNm&amp;keyWord=&amp;stYdFmt=&amp;edYdFmt=&amp;lsClsCd=&amp;cptOfiOrgCd=%EA%B0%9C%EC%9D%B8%EC%A0%95%EB%B3%B4%EB%B3%B4%ED%98%B8%EC%9C%84%EC%9B%90%ED%9A%8C</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1935,22 +1935,22 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>총리령</t>
+          <t>대통령령</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026.05.13</t>
+          <t>2026.06.01</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026.05.20</t>
+          <t>2026.07.13</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1967,17 +1967,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>개인정보 보호법 시행령 일부개정령안 입법예고</t>
+          <t>개인정보보호위원회 직제 시행규칙 일부개정령안 입법예고</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/lawinfo/makingInfo.mo?mid=a10104010000&amp;lawSeq=85978&amp;lawCd=0&amp;lawType=TYPE5&amp;pageCnt=10&amp;currentPage=1&amp;keyField=lmNm&amp;keyWord=&amp;stYdFmt=&amp;edYdFmt=&amp;lsClsCd=&amp;cptOfiOrgCd=%EA%B0%9C%EC%9D%B8%EC%A0%95%EB%B3%B4%EB%B3%B4%ED%98%B8%EC%9C%84%EC%9B%90%ED%9A%8C</t>
+          <t>https://www.moleg.go.kr/lawinfo/makingInfo.mo?mid=a10104010000&amp;lawSeq=86700&amp;lawCd=0&amp;lawType=TYPE5&amp;pageCnt=10&amp;currentPage=1&amp;keyField=lmNm&amp;keyWord=&amp;stYdFmt=&amp;edYdFmt=&amp;lsClsCd=&amp;cptOfiOrgCd=%EA%B0%9C%EC%9D%B8%EC%A0%95%EB%B3%B4%EB%B3%B4%ED%98%B8%EC%9C%84%EC%9B%90%ED%9A%8C</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1987,22 +1987,22 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>대통령령</t>
+          <t>총리령</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026.03.16</t>
+          <t>2026.05.13</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026.04.27</t>
+          <t>2026.05.20</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -2019,17 +2019,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>개인정보보호위원회 직제 시행규칙 일부개정령안 입법예고</t>
+          <t>개인정보 보호법 시행령 일부개정령안 입법예고</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/lawinfo/makingInfo.mo?mid=a10104010000&amp;lawSeq=85936&amp;lawCd=0&amp;lawType=TYPE5&amp;pageCnt=10&amp;currentPage=1&amp;keyField=lmNm&amp;keyWord=&amp;stYdFmt=&amp;edYdFmt=&amp;lsClsCd=&amp;cptOfiOrgCd=%EA%B0%9C%EC%9D%B8%EC%A0%95%EB%B3%B4%EB%B3%B4%ED%98%B8%EC%9C%84%EC%9B%90%ED%9A%8C</t>
+          <t>https://www.moleg.go.kr/lawinfo/makingInfo.mo?mid=a10104010000&amp;lawSeq=85978&amp;lawCd=0&amp;lawType=TYPE5&amp;pageCnt=10&amp;currentPage=1&amp;keyField=lmNm&amp;keyWord=&amp;stYdFmt=&amp;edYdFmt=&amp;lsClsCd=&amp;cptOfiOrgCd=%EA%B0%9C%EC%9D%B8%EC%A0%95%EB%B3%B4%EB%B3%B4%ED%98%B8%EC%9C%84%EC%9B%90%ED%9A%8C</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -2039,22 +2039,22 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>총리령</t>
+          <t>대통령령</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026.03.11</t>
+          <t>2026.03.16</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026.03.18</t>
+          <t>2026.04.27</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -2071,17 +2071,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>개인정보 보호위원회 직제 시행규칙 일부개정령안 입법예고</t>
+          <t>개인정보보호위원회 직제 시행규칙 일부개정령안 입법예고</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/lawinfo/makingInfo.mo?mid=a10104010000&amp;lawSeq=84820&amp;lawCd=0&amp;lawType=TYPE5&amp;pageCnt=10&amp;currentPage=1&amp;keyField=lmNm&amp;keyWord=&amp;stYdFmt=&amp;edYdFmt=&amp;lsClsCd=&amp;cptOfiOrgCd=%EA%B0%9C%EC%9D%B8%EC%A0%95%EB%B3%B4%EB%B3%B4%ED%98%B8%EC%9C%84%EC%9B%90%ED%9A%8C</t>
+          <t>https://www.moleg.go.kr/lawinfo/makingInfo.mo?mid=a10104010000&amp;lawSeq=85936&amp;lawCd=0&amp;lawType=TYPE5&amp;pageCnt=10&amp;currentPage=1&amp;keyField=lmNm&amp;keyWord=&amp;stYdFmt=&amp;edYdFmt=&amp;lsClsCd=&amp;cptOfiOrgCd=%EA%B0%9C%EC%9D%B8%EC%A0%95%EB%B3%B4%EB%B3%B4%ED%98%B8%EC%9C%84%EC%9B%90%ED%9A%8C</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2096,17 +2096,17 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2025.12.16</t>
+          <t>2026.03.11</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2025.12.19</t>
+          <t>2026.03.18</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -2123,17 +2123,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>개인정보 보호법 시행령 일부개정령안 입법예고</t>
+          <t>개인정보 보호위원회 직제 시행규칙 일부개정령안 입법예고</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/lawinfo/makingInfo.mo?mid=a10104010000&amp;lawSeq=83132&amp;lawCd=2000000318612&amp;lawType=TYPE5&amp;pageCnt=10&amp;currentPage=1&amp;keyField=lmNm&amp;keyWord=&amp;stYdFmt=&amp;edYdFmt=&amp;lsClsCd=&amp;cptOfiOrgCd=%EA%B0%9C%EC%9D%B8%EC%A0%95%EB%B3%B4%EB%B3%B4%ED%98%B8%EC%9C%84%EC%9B%90%ED%9A%8C</t>
+          <t>https://www.moleg.go.kr/lawinfo/makingInfo.mo?mid=a10104010000&amp;lawSeq=84820&amp;lawCd=0&amp;lawType=TYPE5&amp;pageCnt=10&amp;currentPage=1&amp;keyField=lmNm&amp;keyWord=&amp;stYdFmt=&amp;edYdFmt=&amp;lsClsCd=&amp;cptOfiOrgCd=%EA%B0%9C%EC%9D%B8%EC%A0%95%EB%B3%B4%EB%B3%B4%ED%98%B8%EC%9C%84%EC%9B%90%ED%9A%8C</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2143,22 +2143,22 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>대통령령</t>
+          <t>총리령</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2025.06.23</t>
+          <t>2025.12.16</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2025.08.04</t>
+          <t>2025.12.19</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2025-06-23</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -2175,7 +2175,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/lawinfo/makingInfo.mo?mid=a10104010000&amp;lawSeq=82960&amp;lawCd=0&amp;lawType=TYPE5&amp;pageCnt=10&amp;currentPage=1&amp;keyField=lmNm&amp;keyWord=&amp;stYdFmt=&amp;edYdFmt=&amp;lsClsCd=&amp;cptOfiOrgCd=%EA%B0%9C%EC%9D%B8%EC%A0%95%EB%B3%B4%EB%B3%B4%ED%98%B8%EC%9C%84%EC%9B%90%ED%9A%8C</t>
+          <t>https://www.moleg.go.kr/lawinfo/makingInfo.mo?mid=a10104010000&amp;lawSeq=83132&amp;lawCd=2000000318612&amp;lawType=TYPE5&amp;pageCnt=10&amp;currentPage=1&amp;keyField=lmNm&amp;keyWord=&amp;stYdFmt=&amp;edYdFmt=&amp;lsClsCd=&amp;cptOfiOrgCd=%EA%B0%9C%EC%9D%B8%EC%A0%95%EB%B3%B4%EB%B3%B4%ED%98%B8%EC%9C%84%EC%9B%90%ED%9A%8C</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2200,17 +2200,17 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2025.05.30</t>
+          <t>2025.06.23</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2025.07.09</t>
+          <t>2025.08.04</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2025-05-30</t>
+          <t>2025-06-23</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -2227,50 +2227,102 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>개인정보 보호법 시행령 일부개정령안 입법예고</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://www.moleg.go.kr/lawinfo/makingInfo.mo?mid=a10104010000&amp;lawSeq=82960&amp;lawCd=0&amp;lawType=TYPE5&amp;pageCnt=10&amp;currentPage=1&amp;keyField=lmNm&amp;keyWord=&amp;stYdFmt=&amp;edYdFmt=&amp;lsClsCd=&amp;cptOfiOrgCd=%EA%B0%9C%EC%9D%B8%EC%A0%95%EB%B3%B4%EB%B3%B4%ED%98%B8%EC%9C%84%EC%9B%90%ED%9A%8C</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>개인정보보호위원회</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>대통령령</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2025.05.30</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2025.07.09</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2025-05-30</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:16.444527+09:00</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:16.444527+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>개인정보 보호위원회 직제 시행규칙 일부개정령안 입법예고</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>https://www.moleg.go.kr/lawinfo/makingInfo.mo?mid=a10104010000&amp;lawSeq=81708&amp;lawCd=2000000315220&amp;lawType=TYPE5&amp;pageCnt=10&amp;currentPage=1&amp;keyField=lmNm&amp;keyWord=&amp;stYdFmt=&amp;edYdFmt=&amp;lsClsCd=&amp;cptOfiOrgCd=%EA%B0%9C%EC%9D%B8%EC%A0%95%EB%B3%B4%EB%B3%B4%ED%98%B8%EC%9C%84%EC%9B%90%ED%9A%8C</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>개인정보보호위원회</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>총리령</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>2025.02.07</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>2025.02.14</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>2025-02-07</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:16.444527+09:00</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:16.444527+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-09-16 15:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,17 +465,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>29141</t>
+          <t>31201</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
+          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -485,7 +485,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -495,39 +495,39 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>27851</t>
+          <t>29141</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
+          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -537,39 +537,39 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>27461</t>
+          <t>27851</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>법제처, 제3회 특별성과 포상 수여</t>
+          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -579,39 +579,39 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>25671</t>
+          <t>27461</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
+          <t>법제처, 제3회 특별성과 포상 수여</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -621,39 +621,39 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>24842</t>
+          <t>25671</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
+          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -663,29 +663,29 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>24841</t>
+          <t>24842</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
+          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -717,27 +717,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>23411</t>
+          <t>24841</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
+          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -747,34 +747,34 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>23231</t>
+          <t>23411</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
+          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>법제자문1담당관</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -789,39 +789,39 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>14381</t>
+          <t>23231</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
+          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>법제자문1담당관</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -831,39 +831,39 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>14121</t>
+          <t>14381</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>법제로 완성하는 국가대전환</t>
+          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -873,39 +873,39 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>12952</t>
+          <t>14121</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
+          <t>법제로 완성하는 국가대전환</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -915,29 +915,29 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12951</t>
+          <t>12952</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
+          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -969,27 +969,27 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>11761</t>
+          <t>12951</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
+          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>법제교육과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -999,34 +999,34 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>11711</t>
+          <t>11761</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
+          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법제교육과</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1041,39 +1041,39 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>11311</t>
+          <t>11711</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>범정부 형벌 합리화 추진단 공식 출범</t>
+          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>파견</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1083,39 +1083,39 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>4471</t>
+          <t>11311</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
+          <t>범정부 형벌 합리화 추진단 공식 출범</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>파견</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1125,39 +1125,39 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1511</t>
+          <t>4471</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
+          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1167,39 +1167,39 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>491</t>
+          <t>1511</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
+          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1209,39 +1209,39 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>491</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
+          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1251,29 +1251,29 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
+          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1305,27 +1305,27 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
+          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1347,27 +1347,27 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
+          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1389,27 +1389,27 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
+          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1431,27 +1431,27 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
+          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1473,27 +1473,27 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
+          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1515,27 +1515,27 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
+          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1557,27 +1557,27 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1599,40 +1599,82 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>대변인실</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>자율주행 규제 합리화, 해외직구 안전 강화 등 국민보호 · 산업지원 새 법령 시행</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150819&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>대변인실</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-09-17 16:20:02 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,27 +465,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>31201</t>
+          <t>31651</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
+          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>경제법제국</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -495,29 +495,29 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>29141</t>
+          <t>31201</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
+          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -527,7 +527,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -537,39 +537,39 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>27851</t>
+          <t>29141</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
+          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -579,39 +579,39 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>27461</t>
+          <t>27851</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>법제처, 제3회 특별성과 포상 수여</t>
+          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -621,39 +621,39 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>25671</t>
+          <t>27461</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
+          <t>법제처, 제3회 특별성과 포상 수여</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -663,39 +663,39 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>24842</t>
+          <t>25671</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
+          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -705,29 +705,29 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>24841</t>
+          <t>24842</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
+          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -759,27 +759,27 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>23411</t>
+          <t>24841</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
+          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -789,34 +789,34 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>23231</t>
+          <t>23411</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
+          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>법제자문1담당관</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -831,39 +831,39 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>14381</t>
+          <t>23231</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
+          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>법제자문1담당관</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -873,39 +873,39 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>14121</t>
+          <t>14381</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>법제로 완성하는 국가대전환</t>
+          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -915,39 +915,39 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12952</t>
+          <t>14121</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
+          <t>법제로 완성하는 국가대전환</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -957,29 +957,29 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12951</t>
+          <t>12952</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
+          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1011,27 +1011,27 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>11761</t>
+          <t>12951</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
+          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>법제교육과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1041,34 +1041,34 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>11711</t>
+          <t>11761</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
+          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법제교육과</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1083,39 +1083,39 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>11311</t>
+          <t>11711</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>범정부 형벌 합리화 추진단 공식 출범</t>
+          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>파견</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1125,39 +1125,39 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>4471</t>
+          <t>11311</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
+          <t>범정부 형벌 합리화 추진단 공식 출범</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>파견</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1167,39 +1167,39 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1511</t>
+          <t>4471</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
+          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1209,39 +1209,39 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>491</t>
+          <t>1511</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
+          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1251,39 +1251,39 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>491</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
+          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1293,29 +1293,29 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
+          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1347,27 +1347,27 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
+          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1389,27 +1389,27 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
+          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1431,27 +1431,27 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
+          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1473,27 +1473,27 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
+          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1515,27 +1515,27 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
+          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1557,27 +1557,27 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
+          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1599,27 +1599,27 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1641,40 +1641,82 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>대변인실</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>자율주행 규제 합리화, 해외직구 안전 강화 등 국민보호 · 산업지원 새 법령 시행</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150819&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>대변인실</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-09-19 14:20:02 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -8920,7 +8920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8968,12 +8968,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026년 개인정보 보호주간(9.28.~10.2.) 포스터 및 앰블럼</t>
+          <t>제6회 개인정보 보호의 날(9.30.) 기념식 개최</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -8983,39 +8983,39 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>20917</t>
+          <t>20920</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20917</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20920</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-09-08 11:31:39.797854+09:00</t>
+          <t>2026-09-19 14:16:49.840552+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-09-08 11:31:39.797854+09:00</t>
+          <t>2026-09-19 14:16:49.840552+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 인증시험(2차) 안내</t>
+          <t>2026년 개인정보 보호주간(9.28.~10.2.) 포스터 및 앰블럼</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9025,39 +9025,39 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>20915</t>
+          <t>20917</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20915</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20917</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-09-03 14:16:40.776731+09:00</t>
+          <t>2026-09-08 11:31:39.797854+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-09-03 14:16:40.776731+09:00</t>
+          <t>2026-09-08 11:31:39.797854+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>개인정보 포털 예방점검에 따른 서비스 중단 안내 (8.13 19:00 ~ 23:00)</t>
+          <t>2026년 개인정보 영향평가 인증시험(2차) 안내</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -9067,39 +9067,39 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>20909</t>
+          <t>20915</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20909</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20915</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-08-10 18:01:43.365104+09:00</t>
+          <t>2026-09-03 14:16:40.776731+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-08-10 18:01:43.365104+09:00</t>
+          <t>2026-09-03 14:16:40.776731+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SKT  휴대폰 본인확인서비스 중단 공지(7.12 01:00 ~ 04:00)</t>
+          <t>개인정보 포털 예방점검에 따른 서비스 중단 안내 (8.13 19:00 ~ 23:00)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -9109,39 +9109,39 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>20908</t>
+          <t>20909</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20908</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20909</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-09 10:02:18.348370+09:00</t>
+          <t>2026-08-10 18:01:43.365104+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-09 10:02:18.348370+09:00</t>
+          <t>2026-08-10 18:01:43.365104+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 전문교육(하반기) 안내</t>
+          <t>SKT  휴대폰 본인확인서비스 중단 공지(7.12 01:00 ~ 04:00)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -9151,39 +9151,39 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>20907</t>
+          <t>20908</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20907</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20908</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-02 13:16:19.799934+09:00</t>
+          <t>2026-07-09 10:02:18.348370+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-02 13:16:19.799934+09:00</t>
+          <t>2026-07-09 10:02:18.348370+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.6.16 (화) 19:00 ~20:00)</t>
+          <t>2026년 개인정보 영향평가 전문교육(하반기) 안내</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -9193,17 +9193,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>20906</t>
+          <t>20907</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20906</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20907</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -9220,12 +9220,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
+          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.6.16 (화) 19:00 ~20:00)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -9235,17 +9235,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>20903</t>
+          <t>20906</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20903</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20906</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -9262,12 +9262,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>개인정보 포털 DB점검에 따른 서비스 중단 안내 (5.26 19:00 ~ 21:00)</t>
+          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -9277,17 +9277,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>20900</t>
+          <t>20903</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20900</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20903</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -9304,12 +9304,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>(복구완료) 외국인 실명확인 서비스 장애 안내(26.05.19 13:47 ~18:50 )</t>
+          <t>개인정보 포털 DB점검에 따른 서비스 중단 안내 (5.26 19:00 ~ 21:00)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -9319,17 +9319,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>20896</t>
+          <t>20900</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20896</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20900</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -9346,12 +9346,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>제3기 가명정보 전문가 풀 모집 공고</t>
+          <t>(복구완료) 외국인 실명확인 서비스 장애 안내(26.05.19 13:47 ~18:50 )</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -9361,17 +9361,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>20895</t>
+          <t>20896</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20895</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20896</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -9388,12 +9388,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>SKT 휴대폰 본인확인서비스 중단 공지(5.10 03:20 ~ 03:25 / 5.12 03:20 ~ 03:25)</t>
+          <t>제3기 가명정보 전문가 풀 모집 공고</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -9403,17 +9403,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>20894</t>
+          <t>20895</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20894</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20895</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -9430,12 +9430,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 인증시험(1차) 안내</t>
+          <t>SKT 휴대폰 본인확인서비스 중단 공지(5.10 03:20 ~ 03:25 / 5.12 03:20 ~ 03:25)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -9445,17 +9445,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>20893</t>
+          <t>20894</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20893</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20894</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -9472,12 +9472,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>본인인증 서비스 장애 발생 공지(2026.04.28(화)15:00 ~ 15:10)</t>
+          <t>2026년 개인정보 영향평가 인증시험(1차) 안내</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -9487,17 +9487,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>20888</t>
+          <t>20893</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20888</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20893</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -9514,12 +9514,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>개인정보 영향평가 전문인력 인증서 발급 및 유효기간 관련 안내</t>
+          <t>본인인증 서비스 장애 발생 공지(2026.04.28(화)15:00 ~ 15:10)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -9529,17 +9529,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>20884</t>
+          <t>20888</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20884</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20888</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -9556,12 +9556,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 계속교육 일정 안내</t>
+          <t>개인정보 영향평가 전문인력 인증서 발급 및 유효기간 관련 안내</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -9571,17 +9571,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>20878</t>
+          <t>20884</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20878</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20884</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -9598,12 +9598,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.4.8 (수) 03:00 ~05:00)</t>
+          <t>2026년 개인정보 영향평가 계속교육 일정 안내</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -9613,17 +9613,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>20875</t>
+          <t>20878</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20875</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20878</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -9640,12 +9640,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내 (2026년 3월 24일(화) 23:00~ 3월 25일(수) 02:00)</t>
+          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.4.8 (수) 03:00 ~05:00)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -9655,17 +9655,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>20874</t>
+          <t>20875</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20874</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20875</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -9682,12 +9682,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.03.24(화)22:00 ~ 2026.03.25(수) 02:00)</t>
+          <t>본인확인 서비스 작업 공지 안내 (2026년 3월 24일(화) 23:00~ 3월 25일(수) 02:00)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -9702,12 +9702,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>20873</t>
+          <t>20874</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20873</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20874</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -9724,12 +9724,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 전문교육(상반기) 안내</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.03.24(화)22:00 ~ 2026.03.25(수) 02:00)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -9744,12 +9744,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>20872</t>
+          <t>20873</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20872</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20873</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -9766,12 +9766,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>외국인 실명확인 서비스 작업 공지 안내</t>
+          <t>2026년 개인정보 영향평가 전문교육(상반기) 안내</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -9781,17 +9781,17 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>20871</t>
+          <t>20872</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20871</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20872</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -9808,12 +9808,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.03.24. (화) 02:00 ~ 04:00)</t>
+          <t>외국인 실명확인 서비스 작업 공지 안내</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -9823,17 +9823,17 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>20870</t>
+          <t>20871</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20870</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20871</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -9850,12 +9850,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.01.22 (목) 22:00 ~2026.01.23 (금) 05:00)</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.03.24. (화) 02:00 ~ 04:00)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -9865,17 +9865,17 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>20868</t>
+          <t>20870</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20868</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20870</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -9892,12 +9892,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.01.21 (수) 19:00 ~21:00)</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.01.22 (목) 22:00 ~2026.01.23 (금) 05:00)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -9907,17 +9907,17 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>20867</t>
+          <t>20868</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20867</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20868</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -9934,12 +9934,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>개인정보 포털 사용자 편의성 설문조사 참여 이벤트 당첨자 발표</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.01.21 (수) 19:00 ~21:00)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -9949,17 +9949,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>20866</t>
+          <t>20867</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20866</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20867</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -9976,12 +9976,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 보호·활용 분야 R&amp;amp;D 사업 신규지원 대상과제 공고(~2.10. 오후 3시)</t>
+          <t>개인정보 포털 사용자 편의성 설문조사 참여 이벤트 당첨자 발표</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -9991,17 +9991,17 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>20865</t>
+          <t>20866</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20865</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20866</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -10018,12 +10018,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.1.12 (월) 05:00 ~06:00)</t>
+          <t>2026년도 개인정보 보호·활용 분야 R&amp;amp;D 사업 신규지원 대상과제 공고(~2.10. 오후 3시)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -10033,17 +10033,17 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>20862</t>
+          <t>20865</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20862</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20865</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -10060,12 +10060,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>「개인정보관리 전문기관 지정 심사위원회」 심사위원 모집 안내 (~12.23. 18시까지)</t>
+          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.1.12 (월) 05:00 ~06:00)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -10075,17 +10075,17 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>20856</t>
+          <t>20862</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20856</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20862</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -10102,12 +10102,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>외국인 본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.17 (수) 16:00 ~17:00)</t>
+          <t>「개인정보관리 전문기관 지정 심사위원회」 심사위원 모집 안내 (~12.23. 18시까지)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -10117,17 +10117,17 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>20855</t>
+          <t>20856</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20855</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20856</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -10144,12 +10144,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.15 (월) 08:00 ~09:00)</t>
+          <t>외국인 본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.17 (수) 16:00 ~17:00)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -10164,12 +10164,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>20854</t>
+          <t>20855</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20854</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20855</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -10186,40 +10186,82 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.15 (월) 08:00 ~09:00)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>관리자</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>20854</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20854</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:16:19.799934+09:00</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:16:19.799934+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>2025년 개인정보 영향평가 인증시험(2차) 안내</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>관리자</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>2025-08-25</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>20837</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20837</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>2026-07-02 13:16:19.799934+09:00</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>2026-07-02 13:16:19.799934+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-09-21 11:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,17 +465,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>31861</t>
+          <t>33082</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
+          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -495,39 +495,39 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>31651</t>
+          <t>31861</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
+          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>경제법제국</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -537,39 +537,39 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>31201</t>
+          <t>31651</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
+          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>경제법제국</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -579,29 +579,29 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>29141</t>
+          <t>31201</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
+          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -621,39 +621,39 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>27851</t>
+          <t>29141</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
+          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -663,39 +663,39 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>27461</t>
+          <t>27851</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>법제처, 제3회 특별성과 포상 수여</t>
+          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -705,39 +705,39 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>25671</t>
+          <t>27461</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
+          <t>법제처, 제3회 특별성과 포상 수여</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -747,39 +747,39 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>24842</t>
+          <t>25671</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
+          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -789,29 +789,29 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>24841</t>
+          <t>24842</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
+          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -843,27 +843,27 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>23411</t>
+          <t>24841</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
+          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -873,34 +873,34 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>23231</t>
+          <t>23411</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
+          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>법제자문1담당관</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -915,39 +915,39 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>14381</t>
+          <t>23231</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
+          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>법제자문1담당관</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -957,39 +957,39 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>14121</t>
+          <t>14381</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>법제로 완성하는 국가대전환</t>
+          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -999,39 +999,39 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>12952</t>
+          <t>14121</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
+          <t>법제로 완성하는 국가대전환</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1041,29 +1041,29 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12951</t>
+          <t>12952</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
+          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1095,27 +1095,27 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>11761</t>
+          <t>12951</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
+          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>법제교육과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1125,34 +1125,34 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>11711</t>
+          <t>11761</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
+          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법제교육과</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1167,39 +1167,39 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>11311</t>
+          <t>11711</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>범정부 형벌 합리화 추진단 공식 출범</t>
+          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>파견</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1209,39 +1209,39 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>4471</t>
+          <t>11311</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
+          <t>범정부 형벌 합리화 추진단 공식 출범</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>파견</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1251,39 +1251,39 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1511</t>
+          <t>4471</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
+          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1293,39 +1293,39 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>491</t>
+          <t>1511</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
+          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1335,39 +1335,39 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>491</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
+          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1377,29 +1377,29 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
+          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1431,27 +1431,27 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
+          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1473,27 +1473,27 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
+          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1515,27 +1515,27 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
+          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1557,27 +1557,27 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
+          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1599,27 +1599,27 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
+          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1641,27 +1641,27 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
+          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1683,27 +1683,27 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1725,40 +1725,82 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>대변인실</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>자율주행 규제 합리화, 해외직구 안전 강화 등 국민보호 · 산업지원 새 법령 시행</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150819&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>대변인실</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-09-21 14:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -9133,7 +9133,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9181,12 +9181,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>제6회 개인정보 보호의 날(9.30.) 기념식 개최</t>
+          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.10.18 (일) 00:00 ~10:00)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -9196,39 +9196,39 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>20920</t>
+          <t>20921</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20920</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20921</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-09-19 14:16:49.840552+09:00</t>
+          <t>2026-09-21 14:16:53.533733+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-09-19 14:16:49.840552+09:00</t>
+          <t>2026-09-21 14:16:53.533733+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026년 개인정보 보호주간(9.28.~10.2.) 포스터 및 앰블럼</t>
+          <t>제6회 개인정보 보호의 날(9.30.) 기념식 개최</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9238,39 +9238,39 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>20917</t>
+          <t>20920</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20917</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20920</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-09-08 11:31:39.797854+09:00</t>
+          <t>2026-09-19 14:16:49.840552+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-09-08 11:31:39.797854+09:00</t>
+          <t>2026-09-19 14:16:49.840552+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 인증시험(2차) 안내</t>
+          <t>2026년 개인정보 보호주간(9.28.~10.2.) 포스터 및 앰블럼</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -9280,39 +9280,39 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>20915</t>
+          <t>20917</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20915</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20917</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-09-03 14:16:40.776731+09:00</t>
+          <t>2026-09-08 11:31:39.797854+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-09-03 14:16:40.776731+09:00</t>
+          <t>2026-09-08 11:31:39.797854+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>개인정보 포털 예방점검에 따른 서비스 중단 안내 (8.13 19:00 ~ 23:00)</t>
+          <t>2026년 개인정보 영향평가 인증시험(2차) 안내</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -9322,39 +9322,39 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>20909</t>
+          <t>20915</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20909</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20915</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-10 18:01:43.365104+09:00</t>
+          <t>2026-09-03 14:16:40.776731+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-08-10 18:01:43.365104+09:00</t>
+          <t>2026-09-03 14:16:40.776731+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SKT  휴대폰 본인확인서비스 중단 공지(7.12 01:00 ~ 04:00)</t>
+          <t>개인정보 포털 예방점검에 따른 서비스 중단 안내 (8.13 19:00 ~ 23:00)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -9364,39 +9364,39 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>20908</t>
+          <t>20909</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20908</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20909</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-09 10:02:18.348370+09:00</t>
+          <t>2026-08-10 18:01:43.365104+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-07-09 10:02:18.348370+09:00</t>
+          <t>2026-08-10 18:01:43.365104+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 전문교육(하반기) 안내</t>
+          <t>SKT  휴대폰 본인확인서비스 중단 공지(7.12 01:00 ~ 04:00)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -9406,39 +9406,39 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>20907</t>
+          <t>20908</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20907</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20908</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-02 13:16:19.799934+09:00</t>
+          <t>2026-07-09 10:02:18.348370+09:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-02 13:16:19.799934+09:00</t>
+          <t>2026-07-09 10:02:18.348370+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.6.16 (화) 19:00 ~20:00)</t>
+          <t>2026년 개인정보 영향평가 전문교육(하반기) 안내</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -9448,17 +9448,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>20906</t>
+          <t>20907</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20906</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20907</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -9475,12 +9475,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
+          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.6.16 (화) 19:00 ~20:00)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -9490,17 +9490,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>20903</t>
+          <t>20906</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20903</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20906</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -9517,12 +9517,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>개인정보 포털 DB점검에 따른 서비스 중단 안내 (5.26 19:00 ~ 21:00)</t>
+          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -9532,17 +9532,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>20900</t>
+          <t>20903</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20900</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20903</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -9559,12 +9559,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>(복구완료) 외국인 실명확인 서비스 장애 안내(26.05.19 13:47 ~18:50 )</t>
+          <t>개인정보 포털 DB점검에 따른 서비스 중단 안내 (5.26 19:00 ~ 21:00)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -9574,17 +9574,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>20896</t>
+          <t>20900</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20896</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20900</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -9601,12 +9601,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>제3기 가명정보 전문가 풀 모집 공고</t>
+          <t>(복구완료) 외국인 실명확인 서비스 장애 안내(26.05.19 13:47 ~18:50 )</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -9616,17 +9616,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>20895</t>
+          <t>20896</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20895</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20896</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -9643,12 +9643,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SKT 휴대폰 본인확인서비스 중단 공지(5.10 03:20 ~ 03:25 / 5.12 03:20 ~ 03:25)</t>
+          <t>제3기 가명정보 전문가 풀 모집 공고</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -9658,17 +9658,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>20894</t>
+          <t>20895</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20894</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20895</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -9685,12 +9685,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 인증시험(1차) 안내</t>
+          <t>SKT 휴대폰 본인확인서비스 중단 공지(5.10 03:20 ~ 03:25 / 5.12 03:20 ~ 03:25)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -9700,17 +9700,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>20893</t>
+          <t>20894</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20893</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20894</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -9727,12 +9727,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>본인인증 서비스 장애 발생 공지(2026.04.28(화)15:00 ~ 15:10)</t>
+          <t>2026년 개인정보 영향평가 인증시험(1차) 안내</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -9742,17 +9742,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>20888</t>
+          <t>20893</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20888</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20893</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -9769,12 +9769,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>개인정보 영향평가 전문인력 인증서 발급 및 유효기간 관련 안내</t>
+          <t>본인인증 서비스 장애 발생 공지(2026.04.28(화)15:00 ~ 15:10)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -9784,17 +9784,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>20884</t>
+          <t>20888</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20884</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20888</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -9811,12 +9811,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 계속교육 일정 안내</t>
+          <t>개인정보 영향평가 전문인력 인증서 발급 및 유효기간 관련 안내</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -9826,17 +9826,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>20878</t>
+          <t>20884</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20878</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20884</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -9853,12 +9853,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.4.8 (수) 03:00 ~05:00)</t>
+          <t>2026년 개인정보 영향평가 계속교육 일정 안내</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -9868,17 +9868,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>20875</t>
+          <t>20878</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20875</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20878</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -9895,12 +9895,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내 (2026년 3월 24일(화) 23:00~ 3월 25일(수) 02:00)</t>
+          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.4.8 (수) 03:00 ~05:00)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -9910,17 +9910,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>20874</t>
+          <t>20875</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20874</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20875</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -9937,12 +9937,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.03.24(화)22:00 ~ 2026.03.25(수) 02:00)</t>
+          <t>본인확인 서비스 작업 공지 안내 (2026년 3월 24일(화) 23:00~ 3월 25일(수) 02:00)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -9957,12 +9957,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>20873</t>
+          <t>20874</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20873</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20874</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -9979,12 +9979,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 전문교육(상반기) 안내</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.03.24(화)22:00 ~ 2026.03.25(수) 02:00)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -9999,12 +9999,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>20872</t>
+          <t>20873</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20872</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20873</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -10021,12 +10021,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>외국인 실명확인 서비스 작업 공지 안내</t>
+          <t>2026년 개인정보 영향평가 전문교육(상반기) 안내</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -10036,17 +10036,17 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>20871</t>
+          <t>20872</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20871</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20872</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -10063,12 +10063,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.03.24. (화) 02:00 ~ 04:00)</t>
+          <t>외국인 실명확인 서비스 작업 공지 안내</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -10078,17 +10078,17 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>20870</t>
+          <t>20871</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20870</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20871</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -10105,12 +10105,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.01.22 (목) 22:00 ~2026.01.23 (금) 05:00)</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.03.24. (화) 02:00 ~ 04:00)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -10120,17 +10120,17 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>20868</t>
+          <t>20870</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20868</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20870</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -10147,12 +10147,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.01.21 (수) 19:00 ~21:00)</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.01.22 (목) 22:00 ~2026.01.23 (금) 05:00)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -10162,17 +10162,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>20867</t>
+          <t>20868</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20867</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20868</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -10189,12 +10189,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>개인정보 포털 사용자 편의성 설문조사 참여 이벤트 당첨자 발표</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.01.21 (수) 19:00 ~21:00)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -10204,17 +10204,17 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>20866</t>
+          <t>20867</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20866</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20867</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -10231,12 +10231,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 보호·활용 분야 R&amp;amp;D 사업 신규지원 대상과제 공고(~2.10. 오후 3시)</t>
+          <t>개인정보 포털 사용자 편의성 설문조사 참여 이벤트 당첨자 발표</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -10246,17 +10246,17 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>20865</t>
+          <t>20866</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20865</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20866</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -10273,12 +10273,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.1.12 (월) 05:00 ~06:00)</t>
+          <t>2026년도 개인정보 보호·활용 분야 R&amp;amp;D 사업 신규지원 대상과제 공고(~2.10. 오후 3시)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -10288,17 +10288,17 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>20862</t>
+          <t>20865</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20862</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20865</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -10315,12 +10315,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>「개인정보관리 전문기관 지정 심사위원회」 심사위원 모집 안내 (~12.23. 18시까지)</t>
+          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.1.12 (월) 05:00 ~06:00)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -10330,17 +10330,17 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>20856</t>
+          <t>20862</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20856</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20862</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -10357,12 +10357,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>외국인 본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.17 (수) 16:00 ~17:00)</t>
+          <t>「개인정보관리 전문기관 지정 심사위원회」 심사위원 모집 안내 (~12.23. 18시까지)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -10372,17 +10372,17 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>20855</t>
+          <t>20856</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20855</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20856</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -10399,12 +10399,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.15 (월) 08:00 ~09:00)</t>
+          <t>외국인 본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.17 (수) 16:00 ~17:00)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -10419,12 +10419,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>20854</t>
+          <t>20855</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20854</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20855</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -10441,40 +10441,82 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.15 (월) 08:00 ~09:00)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>관리자</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>20854</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20854</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:16:19.799934+09:00</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:16:19.799934+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>2025년 개인정보 영향평가 인증시험(2차) 안내</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>관리자</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>2025-08-25</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>20837</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20837</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>2026-07-02 13:16:19.799934+09:00</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>2026-07-02 13:16:19.799934+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-09-22 16:20:02 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,27 +465,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>33082</t>
+          <t>33671</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
+          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>법제조정법제관실</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -495,29 +495,29 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>31861</t>
+          <t>33082</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
+          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -537,39 +537,39 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>31651</t>
+          <t>31861</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
+          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>경제법제국</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -579,39 +579,39 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>31201</t>
+          <t>31651</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
+          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>경제법제국</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -621,29 +621,29 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>29141</t>
+          <t>31201</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
+          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -653,7 +653,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -663,39 +663,39 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>27851</t>
+          <t>29141</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
+          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -705,39 +705,39 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>27461</t>
+          <t>27851</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>법제처, 제3회 특별성과 포상 수여</t>
+          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -747,39 +747,39 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>25671</t>
+          <t>27461</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
+          <t>법제처, 제3회 특별성과 포상 수여</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -789,39 +789,39 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>24842</t>
+          <t>25671</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
+          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -831,29 +831,29 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>24841</t>
+          <t>24842</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
+          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -885,27 +885,27 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>23411</t>
+          <t>24841</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
+          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -915,34 +915,34 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>23231</t>
+          <t>23411</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
+          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>법제자문1담당관</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -957,39 +957,39 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>14381</t>
+          <t>23231</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
+          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>법제자문1담당관</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -999,39 +999,39 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>14121</t>
+          <t>14381</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>법제로 완성하는 국가대전환</t>
+          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1041,39 +1041,39 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12952</t>
+          <t>14121</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
+          <t>법제로 완성하는 국가대전환</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1083,29 +1083,29 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12951</t>
+          <t>12952</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
+          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1137,27 +1137,27 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>11761</t>
+          <t>12951</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
+          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>법제교육과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1167,34 +1167,34 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>11711</t>
+          <t>11761</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
+          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법제교육과</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1209,39 +1209,39 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>11311</t>
+          <t>11711</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>범정부 형벌 합리화 추진단 공식 출범</t>
+          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>파견</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1251,39 +1251,39 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>4471</t>
+          <t>11311</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
+          <t>범정부 형벌 합리화 추진단 공식 출범</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>파견</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1293,39 +1293,39 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1511</t>
+          <t>4471</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
+          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1335,39 +1335,39 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>491</t>
+          <t>1511</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
+          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1377,39 +1377,39 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>491</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
+          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1419,29 +1419,29 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
+          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1473,27 +1473,27 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
+          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1515,27 +1515,27 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
+          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1557,27 +1557,27 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
+          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1599,27 +1599,27 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
+          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1641,27 +1641,27 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
+          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1683,27 +1683,27 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
+          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1725,27 +1725,27 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1767,40 +1767,82 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>대변인실</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>자율주행 규제 합리화, 해외직구 안전 강화 등 국민보호 · 산업지원 새 법령 시행</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150819&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>대변인실</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-09-28 15:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -9403,7 +9403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9451,12 +9451,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.10.18 (일) 00:00 ~10:00)</t>
+          <t>외국인 실명확인 서비스 일시 중단 안내(2026.10.8 (목) 18:00 ~ 10.9.(금) 11:00)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -9466,39 +9466,39 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>20921</t>
+          <t>20922</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20921</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20922</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-09-21 14:16:53.533733+09:00</t>
+          <t>2026-09-28 15:01:57.296841+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-09-21 14:16:53.533733+09:00</t>
+          <t>2026-09-28 15:01:57.296841+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>제6회 개인정보 보호의 날(9.30.) 기념식 개최</t>
+          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.10.18 (일) 00:00 ~10:00)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9508,39 +9508,39 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>20920</t>
+          <t>20921</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20920</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20921</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-09-19 14:16:49.840552+09:00</t>
+          <t>2026-09-21 14:16:53.533733+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-09-19 14:16:49.840552+09:00</t>
+          <t>2026-09-21 14:16:53.533733+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026년 개인정보 보호주간(9.28.~10.2.) 포스터 및 앰블럼</t>
+          <t>제6회 개인정보 보호의 날(9.30.) 기념식 개최</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -9550,39 +9550,39 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>20917</t>
+          <t>20920</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20917</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20920</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-09-08 11:31:39.797854+09:00</t>
+          <t>2026-09-19 14:16:49.840552+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-09-08 11:31:39.797854+09:00</t>
+          <t>2026-09-19 14:16:49.840552+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 인증시험(2차) 안내</t>
+          <t>2026년 개인정보 보호주간(9.28.~10.2.) 포스터 및 앰블럼</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -9592,39 +9592,39 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>20915</t>
+          <t>20917</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20915</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20917</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-03 14:16:40.776731+09:00</t>
+          <t>2026-09-08 11:31:39.797854+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-03 14:16:40.776731+09:00</t>
+          <t>2026-09-08 11:31:39.797854+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>개인정보 포털 예방점검에 따른 서비스 중단 안내 (8.13 19:00 ~ 23:00)</t>
+          <t>2026년 개인정보 영향평가 인증시험(2차) 안내</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -9634,39 +9634,39 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>20909</t>
+          <t>20915</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20909</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20915</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-10 18:01:43.365104+09:00</t>
+          <t>2026-09-03 14:16:40.776731+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-08-10 18:01:43.365104+09:00</t>
+          <t>2026-09-03 14:16:40.776731+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SKT  휴대폰 본인확인서비스 중단 공지(7.12 01:00 ~ 04:00)</t>
+          <t>개인정보 포털 예방점검에 따른 서비스 중단 안내 (8.13 19:00 ~ 23:00)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -9676,39 +9676,39 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>20908</t>
+          <t>20909</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20908</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20909</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-09 10:02:18.348370+09:00</t>
+          <t>2026-08-10 18:01:43.365104+09:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-09 10:02:18.348370+09:00</t>
+          <t>2026-08-10 18:01:43.365104+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 전문교육(하반기) 안내</t>
+          <t>SKT  휴대폰 본인확인서비스 중단 공지(7.12 01:00 ~ 04:00)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -9718,39 +9718,39 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>20907</t>
+          <t>20908</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20907</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20908</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-07-02 13:16:19.799934+09:00</t>
+          <t>2026-07-09 10:02:18.348370+09:00</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-02 13:16:19.799934+09:00</t>
+          <t>2026-07-09 10:02:18.348370+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.6.16 (화) 19:00 ~20:00)</t>
+          <t>2026년 개인정보 영향평가 전문교육(하반기) 안내</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -9760,17 +9760,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>20906</t>
+          <t>20907</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20906</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20907</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -9787,12 +9787,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
+          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.6.16 (화) 19:00 ~20:00)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -9802,17 +9802,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>20903</t>
+          <t>20906</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20903</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20906</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -9829,12 +9829,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>개인정보 포털 DB점검에 따른 서비스 중단 안내 (5.26 19:00 ~ 21:00)</t>
+          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -9844,17 +9844,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>20900</t>
+          <t>20903</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20900</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20903</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -9871,12 +9871,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>(복구완료) 외국인 실명확인 서비스 장애 안내(26.05.19 13:47 ~18:50 )</t>
+          <t>개인정보 포털 DB점검에 따른 서비스 중단 안내 (5.26 19:00 ~ 21:00)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -9886,17 +9886,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>20896</t>
+          <t>20900</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20896</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20900</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -9913,12 +9913,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>제3기 가명정보 전문가 풀 모집 공고</t>
+          <t>(복구완료) 외국인 실명확인 서비스 장애 안내(26.05.19 13:47 ~18:50 )</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -9928,17 +9928,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>20895</t>
+          <t>20896</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20895</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20896</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -9955,12 +9955,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>SKT 휴대폰 본인확인서비스 중단 공지(5.10 03:20 ~ 03:25 / 5.12 03:20 ~ 03:25)</t>
+          <t>제3기 가명정보 전문가 풀 모집 공고</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -9970,17 +9970,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>20894</t>
+          <t>20895</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20894</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20895</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -9997,12 +9997,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 인증시험(1차) 안내</t>
+          <t>SKT 휴대폰 본인확인서비스 중단 공지(5.10 03:20 ~ 03:25 / 5.12 03:20 ~ 03:25)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -10012,17 +10012,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>20893</t>
+          <t>20894</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20893</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20894</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -10039,12 +10039,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>본인인증 서비스 장애 발생 공지(2026.04.28(화)15:00 ~ 15:10)</t>
+          <t>2026년 개인정보 영향평가 인증시험(1차) 안내</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -10054,17 +10054,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>20888</t>
+          <t>20893</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20888</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20893</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -10081,12 +10081,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>개인정보 영향평가 전문인력 인증서 발급 및 유효기간 관련 안내</t>
+          <t>본인인증 서비스 장애 발생 공지(2026.04.28(화)15:00 ~ 15:10)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -10096,17 +10096,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>20884</t>
+          <t>20888</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20884</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20888</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -10123,12 +10123,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 계속교육 일정 안내</t>
+          <t>개인정보 영향평가 전문인력 인증서 발급 및 유효기간 관련 안내</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -10138,17 +10138,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>20878</t>
+          <t>20884</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20878</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20884</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -10165,12 +10165,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.4.8 (수) 03:00 ~05:00)</t>
+          <t>2026년 개인정보 영향평가 계속교육 일정 안내</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -10180,17 +10180,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>20875</t>
+          <t>20878</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20875</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20878</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -10207,12 +10207,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내 (2026년 3월 24일(화) 23:00~ 3월 25일(수) 02:00)</t>
+          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.4.8 (수) 03:00 ~05:00)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -10222,17 +10222,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>20874</t>
+          <t>20875</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20874</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20875</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -10249,12 +10249,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.03.24(화)22:00 ~ 2026.03.25(수) 02:00)</t>
+          <t>본인확인 서비스 작업 공지 안내 (2026년 3월 24일(화) 23:00~ 3월 25일(수) 02:00)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -10269,12 +10269,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>20873</t>
+          <t>20874</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20873</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20874</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -10291,12 +10291,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 전문교육(상반기) 안내</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.03.24(화)22:00 ~ 2026.03.25(수) 02:00)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -10311,12 +10311,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>20872</t>
+          <t>20873</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20872</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20873</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -10333,12 +10333,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>외국인 실명확인 서비스 작업 공지 안내</t>
+          <t>2026년 개인정보 영향평가 전문교육(상반기) 안내</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -10348,17 +10348,17 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>20871</t>
+          <t>20872</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20871</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20872</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -10375,12 +10375,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.03.24. (화) 02:00 ~ 04:00)</t>
+          <t>외국인 실명확인 서비스 작업 공지 안내</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -10390,17 +10390,17 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>20870</t>
+          <t>20871</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20870</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20871</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -10417,12 +10417,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.01.22 (목) 22:00 ~2026.01.23 (금) 05:00)</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.03.24. (화) 02:00 ~ 04:00)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -10432,17 +10432,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>20868</t>
+          <t>20870</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20868</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20870</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -10459,12 +10459,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.01.21 (수) 19:00 ~21:00)</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.01.22 (목) 22:00 ~2026.01.23 (금) 05:00)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -10474,17 +10474,17 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>20867</t>
+          <t>20868</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20867</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20868</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -10501,12 +10501,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>개인정보 포털 사용자 편의성 설문조사 참여 이벤트 당첨자 발표</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.01.21 (수) 19:00 ~21:00)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -10516,17 +10516,17 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>20866</t>
+          <t>20867</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20866</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20867</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -10543,12 +10543,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 보호·활용 분야 R&amp;amp;D 사업 신규지원 대상과제 공고(~2.10. 오후 3시)</t>
+          <t>개인정보 포털 사용자 편의성 설문조사 참여 이벤트 당첨자 발표</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -10558,17 +10558,17 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>20865</t>
+          <t>20866</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20865</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20866</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -10585,12 +10585,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.1.12 (월) 05:00 ~06:00)</t>
+          <t>2026년도 개인정보 보호·활용 분야 R&amp;amp;D 사업 신규지원 대상과제 공고(~2.10. 오후 3시)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -10600,17 +10600,17 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>20862</t>
+          <t>20865</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20862</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20865</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -10627,12 +10627,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>「개인정보관리 전문기관 지정 심사위원회」 심사위원 모집 안내 (~12.23. 18시까지)</t>
+          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.1.12 (월) 05:00 ~06:00)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -10642,17 +10642,17 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>20856</t>
+          <t>20862</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20856</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20862</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -10669,12 +10669,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>외국인 본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.17 (수) 16:00 ~17:00)</t>
+          <t>「개인정보관리 전문기관 지정 심사위원회」 심사위원 모집 안내 (~12.23. 18시까지)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -10684,17 +10684,17 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>20855</t>
+          <t>20856</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20855</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20856</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -10711,12 +10711,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.15 (월) 08:00 ~09:00)</t>
+          <t>외국인 본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.17 (수) 16:00 ~17:00)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -10731,12 +10731,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>20854</t>
+          <t>20855</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20854</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20855</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -10753,40 +10753,82 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.15 (월) 08:00 ~09:00)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>관리자</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>20854</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20854</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:16:19.799934+09:00</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:16:19.799934+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>2025년 개인정보 영향평가 인증시험(2차) 안내</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>관리자</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>2025-08-25</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>20837</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20837</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>2026-07-02 13:16:19.799934+09:00</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>2026-07-02 13:16:19.799934+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-09-29 11:20:02 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,27 +465,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>33671</t>
+          <t>36341</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
+          <t>법제처, AI로 국민과 법의 거리를 좁힌다</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157747&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>법제조정법제관실</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -495,39 +495,39 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-09-22 15:30:19.394844+09:00</t>
+          <t>2026-09-29 10:30:21.085354+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-09-22 15:30:19.394844+09:00</t>
+          <t>2026-09-29 10:30:21.085354+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>33082</t>
+          <t>33671</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
+          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>법제조정법제관실</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -537,29 +537,29 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>31861</t>
+          <t>33082</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
+          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -579,39 +579,39 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>31651</t>
+          <t>31861</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
+          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>경제법제국</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -621,39 +621,39 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>31201</t>
+          <t>31651</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
+          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>경제법제국</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -663,29 +663,29 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>29141</t>
+          <t>31201</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
+          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -705,39 +705,39 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>27851</t>
+          <t>29141</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
+          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -747,39 +747,39 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>27461</t>
+          <t>27851</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>법제처, 제3회 특별성과 포상 수여</t>
+          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -789,39 +789,39 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>25671</t>
+          <t>27461</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
+          <t>법제처, 제3회 특별성과 포상 수여</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -831,39 +831,39 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>24842</t>
+          <t>25671</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
+          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -873,29 +873,29 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>24841</t>
+          <t>24842</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
+          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -927,27 +927,27 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>23411</t>
+          <t>24841</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
+          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -957,34 +957,34 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>23231</t>
+          <t>23411</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
+          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>법제자문1담당관</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -999,39 +999,39 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>14381</t>
+          <t>23231</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
+          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>법제자문1담당관</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1041,39 +1041,39 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>14121</t>
+          <t>14381</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>법제로 완성하는 국가대전환</t>
+          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1083,39 +1083,39 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12952</t>
+          <t>14121</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
+          <t>법제로 완성하는 국가대전환</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1125,29 +1125,29 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12951</t>
+          <t>12952</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
+          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1179,27 +1179,27 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>11761</t>
+          <t>12951</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
+          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>법제교육과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1209,34 +1209,34 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>11711</t>
+          <t>11761</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
+          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법제교육과</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1251,39 +1251,39 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>11311</t>
+          <t>11711</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>범정부 형벌 합리화 추진단 공식 출범</t>
+          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>파견</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1293,39 +1293,39 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>4471</t>
+          <t>11311</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
+          <t>범정부 형벌 합리화 추진단 공식 출범</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>파견</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1335,39 +1335,39 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1511</t>
+          <t>4471</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
+          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1377,39 +1377,39 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>491</t>
+          <t>1511</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
+          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1419,39 +1419,39 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>491</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
+          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1461,29 +1461,29 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
+          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1515,27 +1515,27 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
+          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1557,27 +1557,27 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
+          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1599,27 +1599,27 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
+          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1641,27 +1641,27 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
+          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1683,27 +1683,27 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
+          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1725,27 +1725,27 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
+          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1767,27 +1767,27 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1809,40 +1809,82 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>대변인실</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>자율주행 규제 합리화, 해외직구 안전 강화 등 국민보호 · 산업지원 새 법령 시행</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150819&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>대변인실</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="H35" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-10-01 15:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,22 +465,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>37152</t>
+          <t>37351</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>가상자산 활용 보이스피싱 피해 구제 확대 및 배달앱 원산지 표시 고지 의무화</t>
+          <t>법제처, 알기 쉬운 법령 만들기 20년을 돌아보고 미래를 이야기하다!</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157902&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157915&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -495,29 +495,29 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-01 10:15:19.890918+09:00</t>
+          <t>2026-10-01 15:15:21.104965+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-01 10:15:19.890918+09:00</t>
+          <t>2026-10-01 15:15:21.104965+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>37151</t>
+          <t>37152</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Expanding Voice Phishing Damage Relief Utilizing Virtual Assets and ..</t>
+          <t>가상자산 활용 보이스피싱 피해 구제 확대 및 배달앱 원산지 표시 고지 의무화</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157904&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157902&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -549,17 +549,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>36341</t>
+          <t>37151</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>법제처, AI로 국민과 법의 거리를 좁힌다</t>
+          <t>Expanding Voice Phishing Damage Relief Utilizing Virtual Assets and ..</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157747&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157904&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -569,7 +569,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -579,39 +579,39 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-09-29 10:30:21.085354+09:00</t>
+          <t>2026-10-01 10:15:19.890918+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-09-29 10:30:21.085354+09:00</t>
+          <t>2026-10-01 10:15:19.890918+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>33671</t>
+          <t>36341</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
+          <t>법제처, AI로 국민과 법의 거리를 좁힌다</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157747&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>법제조정법제관실</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -621,39 +621,39 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-22 15:30:19.394844+09:00</t>
+          <t>2026-09-29 10:30:21.085354+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-22 15:30:19.394844+09:00</t>
+          <t>2026-09-29 10:30:21.085354+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>33082</t>
+          <t>33671</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
+          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>법제조정법제관실</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -663,29 +663,29 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>31861</t>
+          <t>33082</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
+          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -705,39 +705,39 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>31651</t>
+          <t>31861</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
+          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>경제법제국</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -747,39 +747,39 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>31201</t>
+          <t>31651</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
+          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>경제법제국</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -789,29 +789,29 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>29141</t>
+          <t>31201</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
+          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -831,39 +831,39 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>27851</t>
+          <t>29141</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
+          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -873,39 +873,39 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>27461</t>
+          <t>27851</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>법제처, 제3회 특별성과 포상 수여</t>
+          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -915,39 +915,39 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>25671</t>
+          <t>27461</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
+          <t>법제처, 제3회 특별성과 포상 수여</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -957,39 +957,39 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>24842</t>
+          <t>25671</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
+          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -999,29 +999,29 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>24841</t>
+          <t>24842</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
+          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1053,27 +1053,27 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>23411</t>
+          <t>24841</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
+          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1083,34 +1083,34 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>23231</t>
+          <t>23411</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
+          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>법제자문1담당관</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1125,39 +1125,39 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>14381</t>
+          <t>23231</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
+          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>법제자문1담당관</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1167,39 +1167,39 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>14121</t>
+          <t>14381</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>법제로 완성하는 국가대전환</t>
+          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1209,39 +1209,39 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12952</t>
+          <t>14121</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
+          <t>법제로 완성하는 국가대전환</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1251,29 +1251,29 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12951</t>
+          <t>12952</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
+          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1305,27 +1305,27 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11761</t>
+          <t>12951</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
+          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>법제교육과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1335,34 +1335,34 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11711</t>
+          <t>11761</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
+          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법제교육과</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1377,39 +1377,39 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11311</t>
+          <t>11711</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>범정부 형벌 합리화 추진단 공식 출범</t>
+          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>파견</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1419,39 +1419,39 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>4471</t>
+          <t>11311</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
+          <t>범정부 형벌 합리화 추진단 공식 출범</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>파견</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1461,39 +1461,39 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1511</t>
+          <t>4471</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
+          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1503,39 +1503,39 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>491</t>
+          <t>1511</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
+          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1545,39 +1545,39 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>491</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
+          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1587,29 +1587,29 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
+          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1641,27 +1641,27 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
+          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1683,27 +1683,27 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
+          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1725,27 +1725,27 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
+          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1767,27 +1767,27 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
+          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1809,27 +1809,27 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
+          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1851,27 +1851,27 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
+          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1893,27 +1893,27 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1935,40 +1935,82 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>대변인실</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>자율주행 규제 합리화, 해외직구 안전 강화 등 국민보호 · 산업지원 새 법령 시행</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150819&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>대변인실</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-10-12 10:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,27 +465,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>37711</t>
+          <t>41651</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>“행정기본법 제정 5주년, 새로운 길을 찾다”</t>
+          <t>법제처, 지방정부 등의 자치법규 입안을 위한 종합안내서 발간</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157976&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158475&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -495,34 +495,34 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-02 14:00:20.071730+09:00</t>
+          <t>2026-10-12 10:00:18.987080+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-02 14:00:20.071730+09:00</t>
+          <t>2026-10-12 10:00:18.987080+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>37581</t>
+          <t>37711</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>국민이 직접 뽑은 ‘대표 알기 쉬운 법령 용어’에 “사위(詐僞) → 거짓/속임수” 등 5개 선정</t>
+          <t>“행정기본법 제정 5주년, 새로운 길을 찾다”</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157972&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157976&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -537,29 +537,29 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-02 10:45:20.519914+09:00</t>
+          <t>2026-10-02 14:00:20.071730+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-02 10:45:20.519914+09:00</t>
+          <t>2026-10-02 14:00:20.071730+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>37351</t>
+          <t>37581</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>법제처, 알기 쉬운 법령 만들기 20년을 돌아보고 미래를 이야기하다!</t>
+          <t>국민이 직접 뽑은 ‘대표 알기 쉬운 법령 용어’에 “사위(詐僞) → 거짓/속임수” 등 5개 선정</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157915&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157972&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -569,7 +569,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -579,34 +579,34 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-01 15:15:21.104965+09:00</t>
+          <t>2026-10-02 10:45:20.519914+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-10-01 15:15:21.104965+09:00</t>
+          <t>2026-10-02 10:45:20.519914+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>37152</t>
+          <t>37351</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>가상자산 활용 보이스피싱 피해 구제 확대 및 배달앱 원산지 표시 고지 의무화</t>
+          <t>법제처, 알기 쉬운 법령 만들기 20년을 돌아보고 미래를 이야기하다!</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157902&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157915&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -621,29 +621,29 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-01 10:15:19.890918+09:00</t>
+          <t>2026-10-01 15:15:21.104965+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-01 10:15:19.890918+09:00</t>
+          <t>2026-10-01 15:15:21.104965+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>37151</t>
+          <t>37152</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Expanding Voice Phishing Damage Relief Utilizing Virtual Assets and ..</t>
+          <t>가상자산 활용 보이스피싱 피해 구제 확대 및 배달앱 원산지 표시 고지 의무화</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157904&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157902&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -675,17 +675,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>36341</t>
+          <t>37151</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>법제처, AI로 국민과 법의 거리를 좁힌다</t>
+          <t>Expanding Voice Phishing Damage Relief Utilizing Virtual Assets and ..</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157747&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157904&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -705,39 +705,39 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-29 10:30:21.085354+09:00</t>
+          <t>2026-10-01 10:15:19.890918+09:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-29 10:30:21.085354+09:00</t>
+          <t>2026-10-01 10:15:19.890918+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>33671</t>
+          <t>36341</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
+          <t>법제처, AI로 국민과 법의 거리를 좁힌다</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157747&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>법제조정법제관실</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -747,39 +747,39 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-09-22 15:30:19.394844+09:00</t>
+          <t>2026-09-29 10:30:21.085354+09:00</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-22 15:30:19.394844+09:00</t>
+          <t>2026-09-29 10:30:21.085354+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>33082</t>
+          <t>33671</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
+          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>법제조정법제관실</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -789,29 +789,29 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>31861</t>
+          <t>33082</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
+          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -831,39 +831,39 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>31651</t>
+          <t>31861</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
+          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>경제법제국</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -873,39 +873,39 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>31201</t>
+          <t>31651</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
+          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>경제법제국</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -915,29 +915,29 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>29141</t>
+          <t>31201</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
+          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -957,39 +957,39 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>27851</t>
+          <t>29141</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
+          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -999,39 +999,39 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>27461</t>
+          <t>27851</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>법제처, 제3회 특별성과 포상 수여</t>
+          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1041,39 +1041,39 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>25671</t>
+          <t>27461</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
+          <t>법제처, 제3회 특별성과 포상 수여</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1083,39 +1083,39 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>24842</t>
+          <t>25671</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
+          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1125,29 +1125,29 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>24841</t>
+          <t>24842</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
+          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1179,27 +1179,27 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>23411</t>
+          <t>24841</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
+          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1209,34 +1209,34 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>23231</t>
+          <t>23411</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
+          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>법제자문1담당관</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1251,39 +1251,39 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>14381</t>
+          <t>23231</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
+          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>법제자문1담당관</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1293,39 +1293,39 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>14121</t>
+          <t>14381</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>법제로 완성하는 국가대전환</t>
+          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1335,39 +1335,39 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12952</t>
+          <t>14121</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
+          <t>법제로 완성하는 국가대전환</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1377,29 +1377,29 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12951</t>
+          <t>12952</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
+          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1431,27 +1431,27 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11761</t>
+          <t>12951</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
+          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>법제교육과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1461,34 +1461,34 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>11711</t>
+          <t>11761</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
+          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법제교육과</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1503,39 +1503,39 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>11311</t>
+          <t>11711</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>범정부 형벌 합리화 추진단 공식 출범</t>
+          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>파견</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1545,39 +1545,39 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>4471</t>
+          <t>11311</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
+          <t>범정부 형벌 합리화 추진단 공식 출범</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>파견</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1587,39 +1587,39 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1511</t>
+          <t>4471</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
+          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1629,39 +1629,39 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>491</t>
+          <t>1511</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
+          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1671,39 +1671,39 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>491</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
+          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1713,29 +1713,29 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
+          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1767,27 +1767,27 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
+          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1809,27 +1809,27 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
+          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1851,27 +1851,27 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
+          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1893,27 +1893,27 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
+          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1935,27 +1935,27 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
+          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1977,27 +1977,27 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
+          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2019,27 +2019,27 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2061,40 +2061,82 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>대변인실</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>자율주행 규제 합리화, 해외직구 안전 강화 등 국민보호 · 산업지원 새 법령 시행</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150819&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>대변인실</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="H41" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-10-13 14:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -10609,7 +10609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10657,12 +10657,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>외국인 실명확인 서비스 일시 중단 안내(2026.10.8 (목) 18:00 ~ 10.9.(금) 11:00)</t>
+          <t>개인정보 유출신고시스템 작업에 따른 서비스 일시 중단 및 대체 신고 방법 안내</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -10672,39 +10672,39 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>20922</t>
+          <t>20924</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20922</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20924</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-09-28 15:01:57.296841+09:00</t>
+          <t>2026-10-13 13:31:56.172770+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-09-28 15:01:57.296841+09:00</t>
+          <t>2026-10-13 13:31:56.172770+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.10.18 (일) 00:00 ~10:00)</t>
+          <t>외국인 실명확인 서비스 일시 중단 안내(2026.10.8 (목) 18:00 ~ 10.9.(금) 11:00)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10714,39 +10714,39 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>20921</t>
+          <t>20922</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20921</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20922</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-09-21 14:16:53.533733+09:00</t>
+          <t>2026-09-28 15:01:57.296841+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-09-21 14:16:53.533733+09:00</t>
+          <t>2026-09-28 15:01:57.296841+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>제6회 개인정보 보호의 날(9.30.) 기념식 개최</t>
+          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.10.18 (일) 00:00 ~10:00)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -10756,39 +10756,39 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>20920</t>
+          <t>20921</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20920</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20921</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-09-19 14:16:49.840552+09:00</t>
+          <t>2026-09-21 14:16:53.533733+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-09-19 14:16:49.840552+09:00</t>
+          <t>2026-09-21 14:16:53.533733+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026년 개인정보 보호주간(9.28.~10.2.) 포스터 및 앰블럼</t>
+          <t>제6회 개인정보 보호의 날(9.30.) 기념식 개최</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -10798,39 +10798,39 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>20917</t>
+          <t>20920</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20917</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20920</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-08 11:31:39.797854+09:00</t>
+          <t>2026-09-19 14:16:49.840552+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-08 11:31:39.797854+09:00</t>
+          <t>2026-09-19 14:16:49.840552+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 인증시험(2차) 안내</t>
+          <t>2026년 개인정보 보호주간(9.28.~10.2.) 포스터 및 앰블럼</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -10840,39 +10840,39 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>20915</t>
+          <t>20917</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20915</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20917</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-03 14:16:40.776731+09:00</t>
+          <t>2026-09-08 11:31:39.797854+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-03 14:16:40.776731+09:00</t>
+          <t>2026-09-08 11:31:39.797854+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>개인정보 포털 예방점검에 따른 서비스 중단 안내 (8.13 19:00 ~ 23:00)</t>
+          <t>2026년 개인정보 영향평가 인증시험(2차) 안내</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -10882,39 +10882,39 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>20909</t>
+          <t>20915</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20909</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20915</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-10 18:01:43.365104+09:00</t>
+          <t>2026-09-03 14:16:40.776731+09:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-08-10 18:01:43.365104+09:00</t>
+          <t>2026-09-03 14:16:40.776731+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SKT  휴대폰 본인확인서비스 중단 공지(7.12 01:00 ~ 04:00)</t>
+          <t>개인정보 포털 예방점검에 따른 서비스 중단 안내 (8.13 19:00 ~ 23:00)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -10924,39 +10924,39 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>20908</t>
+          <t>20909</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20908</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20909</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-07-09 10:02:18.348370+09:00</t>
+          <t>2026-08-10 18:01:43.365104+09:00</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-07-09 10:02:18.348370+09:00</t>
+          <t>2026-08-10 18:01:43.365104+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 전문교육(하반기) 안내</t>
+          <t>SKT  휴대폰 본인확인서비스 중단 공지(7.12 01:00 ~ 04:00)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -10966,39 +10966,39 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>20907</t>
+          <t>20908</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20907</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20908</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-07-02 13:16:19.799934+09:00</t>
+          <t>2026-07-09 10:02:18.348370+09:00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-02 13:16:19.799934+09:00</t>
+          <t>2026-07-09 10:02:18.348370+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.6.16 (화) 19:00 ~20:00)</t>
+          <t>2026년 개인정보 영향평가 전문교육(하반기) 안내</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -11008,17 +11008,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>20906</t>
+          <t>20907</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20906</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20907</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -11035,12 +11035,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
+          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.6.16 (화) 19:00 ~20:00)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -11050,17 +11050,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>20903</t>
+          <t>20906</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20903</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20906</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -11077,12 +11077,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>개인정보 포털 DB점검에 따른 서비스 중단 안내 (5.26 19:00 ~ 21:00)</t>
+          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -11092,17 +11092,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>20900</t>
+          <t>20903</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20900</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20903</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -11119,12 +11119,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>(복구완료) 외국인 실명확인 서비스 장애 안내(26.05.19 13:47 ~18:50 )</t>
+          <t>개인정보 포털 DB점검에 따른 서비스 중단 안내 (5.26 19:00 ~ 21:00)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -11134,17 +11134,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>20896</t>
+          <t>20900</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20896</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20900</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -11161,12 +11161,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>제3기 가명정보 전문가 풀 모집 공고</t>
+          <t>(복구완료) 외국인 실명확인 서비스 장애 안내(26.05.19 13:47 ~18:50 )</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -11176,17 +11176,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>20895</t>
+          <t>20896</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20895</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20896</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -11203,12 +11203,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SKT 휴대폰 본인확인서비스 중단 공지(5.10 03:20 ~ 03:25 / 5.12 03:20 ~ 03:25)</t>
+          <t>제3기 가명정보 전문가 풀 모집 공고</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -11218,17 +11218,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>20894</t>
+          <t>20895</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20894</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20895</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -11245,12 +11245,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 인증시험(1차) 안내</t>
+          <t>SKT 휴대폰 본인확인서비스 중단 공지(5.10 03:20 ~ 03:25 / 5.12 03:20 ~ 03:25)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -11260,17 +11260,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>20893</t>
+          <t>20894</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20893</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20894</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -11287,12 +11287,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>본인인증 서비스 장애 발생 공지(2026.04.28(화)15:00 ~ 15:10)</t>
+          <t>2026년 개인정보 영향평가 인증시험(1차) 안내</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -11302,17 +11302,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>20888</t>
+          <t>20893</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20888</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20893</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -11329,12 +11329,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>개인정보 영향평가 전문인력 인증서 발급 및 유효기간 관련 안내</t>
+          <t>본인인증 서비스 장애 발생 공지(2026.04.28(화)15:00 ~ 15:10)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -11344,17 +11344,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>20884</t>
+          <t>20888</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20884</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20888</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -11371,12 +11371,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 계속교육 일정 안내</t>
+          <t>개인정보 영향평가 전문인력 인증서 발급 및 유효기간 관련 안내</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -11386,17 +11386,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>20878</t>
+          <t>20884</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20878</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20884</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -11413,12 +11413,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.4.8 (수) 03:00 ~05:00)</t>
+          <t>2026년 개인정보 영향평가 계속교육 일정 안내</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -11428,17 +11428,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>20875</t>
+          <t>20878</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20875</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20878</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -11455,12 +11455,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내 (2026년 3월 24일(화) 23:00~ 3월 25일(수) 02:00)</t>
+          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.4.8 (수) 03:00 ~05:00)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -11470,17 +11470,17 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>20874</t>
+          <t>20875</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20874</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20875</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -11497,12 +11497,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.03.24(화)22:00 ~ 2026.03.25(수) 02:00)</t>
+          <t>본인확인 서비스 작업 공지 안내 (2026년 3월 24일(화) 23:00~ 3월 25일(수) 02:00)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -11517,12 +11517,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>20873</t>
+          <t>20874</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20873</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20874</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -11539,12 +11539,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 전문교육(상반기) 안내</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.03.24(화)22:00 ~ 2026.03.25(수) 02:00)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -11559,12 +11559,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>20872</t>
+          <t>20873</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20872</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20873</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -11581,12 +11581,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>외국인 실명확인 서비스 작업 공지 안내</t>
+          <t>2026년 개인정보 영향평가 전문교육(상반기) 안내</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -11596,17 +11596,17 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>20871</t>
+          <t>20872</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20871</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20872</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -11623,12 +11623,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.03.24. (화) 02:00 ~ 04:00)</t>
+          <t>외국인 실명확인 서비스 작업 공지 안내</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -11638,17 +11638,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>20870</t>
+          <t>20871</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20870</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20871</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -11665,12 +11665,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.01.22 (목) 22:00 ~2026.01.23 (금) 05:00)</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.03.24. (화) 02:00 ~ 04:00)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -11680,17 +11680,17 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>20868</t>
+          <t>20870</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20868</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20870</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -11707,12 +11707,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.01.21 (수) 19:00 ~21:00)</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.01.22 (목) 22:00 ~2026.01.23 (금) 05:00)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -11722,17 +11722,17 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>20867</t>
+          <t>20868</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20867</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20868</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -11749,12 +11749,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>개인정보 포털 사용자 편의성 설문조사 참여 이벤트 당첨자 발표</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.01.21 (수) 19:00 ~21:00)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -11764,17 +11764,17 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>20866</t>
+          <t>20867</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20866</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20867</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -11791,12 +11791,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 보호·활용 분야 R&amp;amp;D 사업 신규지원 대상과제 공고(~2.10. 오후 3시)</t>
+          <t>개인정보 포털 사용자 편의성 설문조사 참여 이벤트 당첨자 발표</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -11806,17 +11806,17 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>20865</t>
+          <t>20866</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20865</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20866</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -11833,12 +11833,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.1.12 (월) 05:00 ~06:00)</t>
+          <t>2026년도 개인정보 보호·활용 분야 R&amp;amp;D 사업 신규지원 대상과제 공고(~2.10. 오후 3시)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -11848,17 +11848,17 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>20862</t>
+          <t>20865</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20862</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20865</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -11875,12 +11875,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>「개인정보관리 전문기관 지정 심사위원회」 심사위원 모집 안내 (~12.23. 18시까지)</t>
+          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.1.12 (월) 05:00 ~06:00)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -11890,17 +11890,17 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>20856</t>
+          <t>20862</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20856</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20862</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -11917,12 +11917,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>외국인 본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.17 (수) 16:00 ~17:00)</t>
+          <t>「개인정보관리 전문기관 지정 심사위원회」 심사위원 모집 안내 (~12.23. 18시까지)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -11932,17 +11932,17 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>20855</t>
+          <t>20856</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20855</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20856</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -11959,12 +11959,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.15 (월) 08:00 ~09:00)</t>
+          <t>외국인 본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.17 (수) 16:00 ~17:00)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -11979,12 +11979,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>20854</t>
+          <t>20855</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20854</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20855</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -12001,40 +12001,82 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.15 (월) 08:00 ~09:00)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>관리자</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>20854</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20854</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:16:19.799934+09:00</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:16:19.799934+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>2025년 개인정보 영향평가 인증시험(2차) 안내</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>관리자</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>2025-08-25</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>20837</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20837</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>2026-07-02 13:16:19.799934+09:00</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="H35" t="inlineStr">
         <is>
           <t>2026-07-02 13:16:19.799934+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-10-20 11:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -10894,7 +10894,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10942,12 +10942,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>개인정보 유출신고시스템 작업에 따른 서비스 일시 중단 및 대체 신고 방법 안내</t>
+          <t>외국인 실명확인 서비스 일시 중단 안내(2026.10.24 (토) 22:00 ~ 10.25.(일) 04:00)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -10957,39 +10957,39 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>20924</t>
+          <t>20927</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20924</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20927</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-13 13:31:56.172770+09:00</t>
+          <t>2026-10-20 11:01:57.312740+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-13 13:31:56.172770+09:00</t>
+          <t>2026-10-20 11:01:57.312740+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>외국인 실명확인 서비스 일시 중단 안내(2026.10.8 (목) 18:00 ~ 10.9.(금) 11:00)</t>
+          <t>개인정보 유출신고시스템 작업에 따른 서비스 일시 중단 및 대체 신고 방법 안내</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10999,39 +10999,39 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>20922</t>
+          <t>20924</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20922</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20924</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-09-28 15:01:57.296841+09:00</t>
+          <t>2026-10-13 13:31:56.172770+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-09-28 15:01:57.296841+09:00</t>
+          <t>2026-10-13 13:31:56.172770+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.10.18 (일) 00:00 ~10:00)</t>
+          <t>외국인 실명확인 서비스 일시 중단 안내(2026.10.8 (목) 18:00 ~ 10.9.(금) 11:00)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -11041,39 +11041,39 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>20921</t>
+          <t>20922</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20921</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20922</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-09-21 14:16:53.533733+09:00</t>
+          <t>2026-09-28 15:01:57.296841+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-09-21 14:16:53.533733+09:00</t>
+          <t>2026-09-28 15:01:57.296841+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>제6회 개인정보 보호의 날(9.30.) 기념식 개최</t>
+          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.10.18 (일) 00:00 ~10:00)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -11083,39 +11083,39 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>20920</t>
+          <t>20921</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20920</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20921</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-19 14:16:49.840552+09:00</t>
+          <t>2026-09-21 14:16:53.533733+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-19 14:16:49.840552+09:00</t>
+          <t>2026-09-21 14:16:53.533733+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026년 개인정보 보호주간(9.28.~10.2.) 포스터 및 앰블럼</t>
+          <t>제6회 개인정보 보호의 날(9.30.) 기념식 개최</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -11125,39 +11125,39 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>20917</t>
+          <t>20920</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20917</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20920</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-08 11:31:39.797854+09:00</t>
+          <t>2026-09-19 14:16:49.840552+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-08 11:31:39.797854+09:00</t>
+          <t>2026-09-19 14:16:49.840552+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 인증시험(2차) 안내</t>
+          <t>2026년 개인정보 보호주간(9.28.~10.2.) 포스터 및 앰블럼</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -11167,39 +11167,39 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>20915</t>
+          <t>20917</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20915</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20917</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-03 14:16:40.776731+09:00</t>
+          <t>2026-09-08 11:31:39.797854+09:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-03 14:16:40.776731+09:00</t>
+          <t>2026-09-08 11:31:39.797854+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>개인정보 포털 예방점검에 따른 서비스 중단 안내 (8.13 19:00 ~ 23:00)</t>
+          <t>2026년 개인정보 영향평가 인증시험(2차) 안내</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -11209,39 +11209,39 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>20909</t>
+          <t>20915</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20909</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20915</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-08-10 18:01:43.365104+09:00</t>
+          <t>2026-09-03 14:16:40.776731+09:00</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-08-10 18:01:43.365104+09:00</t>
+          <t>2026-09-03 14:16:40.776731+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SKT  휴대폰 본인확인서비스 중단 공지(7.12 01:00 ~ 04:00)</t>
+          <t>개인정보 포털 예방점검에 따른 서비스 중단 안내 (8.13 19:00 ~ 23:00)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -11251,39 +11251,39 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>20908</t>
+          <t>20909</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20908</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20909</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-07-09 10:02:18.348370+09:00</t>
+          <t>2026-08-10 18:01:43.365104+09:00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-09 10:02:18.348370+09:00</t>
+          <t>2026-08-10 18:01:43.365104+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 전문교육(하반기) 안내</t>
+          <t>SKT  휴대폰 본인확인서비스 중단 공지(7.12 01:00 ~ 04:00)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -11293,39 +11293,39 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>20907</t>
+          <t>20908</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20907</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20908</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-07-02 13:16:19.799934+09:00</t>
+          <t>2026-07-09 10:02:18.348370+09:00</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-02 13:16:19.799934+09:00</t>
+          <t>2026-07-09 10:02:18.348370+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.6.16 (화) 19:00 ~20:00)</t>
+          <t>2026년 개인정보 영향평가 전문교육(하반기) 안내</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -11335,17 +11335,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>20906</t>
+          <t>20907</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20906</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20907</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -11362,12 +11362,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
+          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.6.16 (화) 19:00 ~20:00)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -11377,17 +11377,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>20903</t>
+          <t>20906</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20903</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20906</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -11404,12 +11404,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>개인정보 포털 DB점검에 따른 서비스 중단 안내 (5.26 19:00 ~ 21:00)</t>
+          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -11419,17 +11419,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>20900</t>
+          <t>20903</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20900</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20903</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -11446,12 +11446,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>(복구완료) 외국인 실명확인 서비스 장애 안내(26.05.19 13:47 ~18:50 )</t>
+          <t>개인정보 포털 DB점검에 따른 서비스 중단 안내 (5.26 19:00 ~ 21:00)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -11461,17 +11461,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>20896</t>
+          <t>20900</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20896</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20900</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -11488,12 +11488,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>제3기 가명정보 전문가 풀 모집 공고</t>
+          <t>(복구완료) 외국인 실명확인 서비스 장애 안내(26.05.19 13:47 ~18:50 )</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -11503,17 +11503,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>20895</t>
+          <t>20896</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20895</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20896</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -11530,12 +11530,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>SKT 휴대폰 본인확인서비스 중단 공지(5.10 03:20 ~ 03:25 / 5.12 03:20 ~ 03:25)</t>
+          <t>제3기 가명정보 전문가 풀 모집 공고</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -11545,17 +11545,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>20894</t>
+          <t>20895</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20894</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20895</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -11572,12 +11572,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 인증시험(1차) 안내</t>
+          <t>SKT 휴대폰 본인확인서비스 중단 공지(5.10 03:20 ~ 03:25 / 5.12 03:20 ~ 03:25)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -11587,17 +11587,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>20893</t>
+          <t>20894</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20893</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20894</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -11614,12 +11614,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>본인인증 서비스 장애 발생 공지(2026.04.28(화)15:00 ~ 15:10)</t>
+          <t>2026년 개인정보 영향평가 인증시험(1차) 안내</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -11629,17 +11629,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>20888</t>
+          <t>20893</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20888</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20893</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -11656,12 +11656,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>개인정보 영향평가 전문인력 인증서 발급 및 유효기간 관련 안내</t>
+          <t>본인인증 서비스 장애 발생 공지(2026.04.28(화)15:00 ~ 15:10)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -11671,17 +11671,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>20884</t>
+          <t>20888</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20884</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20888</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -11698,12 +11698,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 계속교육 일정 안내</t>
+          <t>개인정보 영향평가 전문인력 인증서 발급 및 유효기간 관련 안내</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -11713,17 +11713,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>20878</t>
+          <t>20884</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20878</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20884</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -11740,12 +11740,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.4.8 (수) 03:00 ~05:00)</t>
+          <t>2026년 개인정보 영향평가 계속교육 일정 안내</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -11755,17 +11755,17 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>20875</t>
+          <t>20878</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20875</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20878</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -11782,12 +11782,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내 (2026년 3월 24일(화) 23:00~ 3월 25일(수) 02:00)</t>
+          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.4.8 (수) 03:00 ~05:00)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -11797,17 +11797,17 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>20874</t>
+          <t>20875</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20874</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20875</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -11824,12 +11824,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.03.24(화)22:00 ~ 2026.03.25(수) 02:00)</t>
+          <t>본인확인 서비스 작업 공지 안내 (2026년 3월 24일(화) 23:00~ 3월 25일(수) 02:00)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -11844,12 +11844,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>20873</t>
+          <t>20874</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20873</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20874</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -11866,12 +11866,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 전문교육(상반기) 안내</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.03.24(화)22:00 ~ 2026.03.25(수) 02:00)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -11886,12 +11886,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>20872</t>
+          <t>20873</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20872</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20873</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -11908,12 +11908,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>외국인 실명확인 서비스 작업 공지 안내</t>
+          <t>2026년 개인정보 영향평가 전문교육(상반기) 안내</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -11923,17 +11923,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>20871</t>
+          <t>20872</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20871</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20872</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -11950,12 +11950,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.03.24. (화) 02:00 ~ 04:00)</t>
+          <t>외국인 실명확인 서비스 작업 공지 안내</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -11965,17 +11965,17 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>20870</t>
+          <t>20871</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20870</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20871</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -11992,12 +11992,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.01.22 (목) 22:00 ~2026.01.23 (금) 05:00)</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.03.24. (화) 02:00 ~ 04:00)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -12007,17 +12007,17 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>20868</t>
+          <t>20870</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20868</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20870</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -12034,12 +12034,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.01.21 (수) 19:00 ~21:00)</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.01.22 (목) 22:00 ~2026.01.23 (금) 05:00)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -12049,17 +12049,17 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>20867</t>
+          <t>20868</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20867</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20868</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -12076,12 +12076,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>개인정보 포털 사용자 편의성 설문조사 참여 이벤트 당첨자 발표</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.01.21 (수) 19:00 ~21:00)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -12091,17 +12091,17 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>20866</t>
+          <t>20867</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20866</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20867</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -12118,12 +12118,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 보호·활용 분야 R&amp;amp;D 사업 신규지원 대상과제 공고(~2.10. 오후 3시)</t>
+          <t>개인정보 포털 사용자 편의성 설문조사 참여 이벤트 당첨자 발표</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -12133,17 +12133,17 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>20865</t>
+          <t>20866</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20865</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20866</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -12160,12 +12160,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.1.12 (월) 05:00 ~06:00)</t>
+          <t>2026년도 개인정보 보호·활용 분야 R&amp;amp;D 사업 신규지원 대상과제 공고(~2.10. 오후 3시)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -12175,17 +12175,17 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>20862</t>
+          <t>20865</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20862</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20865</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -12202,12 +12202,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>「개인정보관리 전문기관 지정 심사위원회」 심사위원 모집 안내 (~12.23. 18시까지)</t>
+          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.1.12 (월) 05:00 ~06:00)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -12217,17 +12217,17 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>20856</t>
+          <t>20862</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20856</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20862</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -12244,12 +12244,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>외국인 본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.17 (수) 16:00 ~17:00)</t>
+          <t>「개인정보관리 전문기관 지정 심사위원회」 심사위원 모집 안내 (~12.23. 18시까지)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -12259,17 +12259,17 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>20855</t>
+          <t>20856</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20855</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20856</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -12286,12 +12286,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.15 (월) 08:00 ~09:00)</t>
+          <t>외국인 본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.17 (수) 16:00 ~17:00)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -12306,12 +12306,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>20854</t>
+          <t>20855</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20854</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20855</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -12328,40 +12328,82 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.15 (월) 08:00 ~09:00)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>관리자</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>20854</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20854</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:16:19.799934+09:00</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:16:19.799934+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>2025년 개인정보 영향평가 인증시험(2차) 안내</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>관리자</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>2025-08-25</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>20837</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20837</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>2026-07-02 13:16:19.799934+09:00</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="H36" t="inlineStr">
         <is>
           <t>2026-07-02 13:16:19.799934+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-10-20 15:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,27 +465,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>41651</t>
+          <t>45121</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>법제처, 지방정부 등의 자치법규 입안을 위한 종합안내서 발간</t>
+          <t>국민의 생애주기에 맞춘 생활법령정보 서비스 발전 방안 논의</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158475&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158862&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -495,39 +495,39 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-12 10:00:18.987080+09:00</t>
+          <t>2026-10-20 14:45:19.906187+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-12 10:00:18.987080+09:00</t>
+          <t>2026-10-20 14:45:19.906187+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>37711</t>
+          <t>41651</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>“행정기본법 제정 5주년, 새로운 길을 찾다”</t>
+          <t>법제처, 지방정부 등의 자치법규 입안을 위한 종합안내서 발간</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157976&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158475&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -537,34 +537,34 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-02 14:00:20.071730+09:00</t>
+          <t>2026-10-12 10:00:18.987080+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-02 14:00:20.071730+09:00</t>
+          <t>2026-10-12 10:00:18.987080+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>37581</t>
+          <t>37711</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>국민이 직접 뽑은 ‘대표 알기 쉬운 법령 용어’에 “사위(詐僞) → 거짓/속임수” 등 5개 선정</t>
+          <t>“행정기본법 제정 5주년, 새로운 길을 찾다”</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157972&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157976&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -579,29 +579,29 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-02 10:45:20.519914+09:00</t>
+          <t>2026-10-02 14:00:20.071730+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-10-02 10:45:20.519914+09:00</t>
+          <t>2026-10-02 14:00:20.071730+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>37351</t>
+          <t>37581</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>법제처, 알기 쉬운 법령 만들기 20년을 돌아보고 미래를 이야기하다!</t>
+          <t>국민이 직접 뽑은 ‘대표 알기 쉬운 법령 용어’에 “사위(詐僞) → 거짓/속임수” 등 5개 선정</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157915&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157972&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -621,34 +621,34 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-01 15:15:21.104965+09:00</t>
+          <t>2026-10-02 10:45:20.519914+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-01 15:15:21.104965+09:00</t>
+          <t>2026-10-02 10:45:20.519914+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>37152</t>
+          <t>37351</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>가상자산 활용 보이스피싱 피해 구제 확대 및 배달앱 원산지 표시 고지 의무화</t>
+          <t>법제처, 알기 쉬운 법령 만들기 20년을 돌아보고 미래를 이야기하다!</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157902&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157915&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -663,29 +663,29 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-01 10:15:19.890918+09:00</t>
+          <t>2026-10-01 15:15:21.104965+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-01 10:15:19.890918+09:00</t>
+          <t>2026-10-01 15:15:21.104965+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>37151</t>
+          <t>37152</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Expanding Voice Phishing Damage Relief Utilizing Virtual Assets and ..</t>
+          <t>가상자산 활용 보이스피싱 피해 구제 확대 및 배달앱 원산지 표시 고지 의무화</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157904&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157902&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -717,17 +717,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>36341</t>
+          <t>37151</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>법제처, AI로 국민과 법의 거리를 좁힌다</t>
+          <t>Expanding Voice Phishing Damage Relief Utilizing Virtual Assets and ..</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157747&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157904&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -737,7 +737,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -747,39 +747,39 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-09-29 10:30:21.085354+09:00</t>
+          <t>2026-10-01 10:15:19.890918+09:00</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-29 10:30:21.085354+09:00</t>
+          <t>2026-10-01 10:15:19.890918+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>33671</t>
+          <t>36341</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
+          <t>법제처, AI로 국민과 법의 거리를 좁힌다</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157747&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>법제조정법제관실</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -789,39 +789,39 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-09-22 15:30:19.394844+09:00</t>
+          <t>2026-09-29 10:30:21.085354+09:00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-22 15:30:19.394844+09:00</t>
+          <t>2026-09-29 10:30:21.085354+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>33082</t>
+          <t>33671</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
+          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>법제조정법제관실</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -831,29 +831,29 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>31861</t>
+          <t>33082</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
+          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -873,39 +873,39 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>31651</t>
+          <t>31861</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
+          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>경제법제국</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -915,39 +915,39 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>31201</t>
+          <t>31651</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
+          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>경제법제국</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -957,29 +957,29 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>29141</t>
+          <t>31201</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
+          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -989,7 +989,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -999,39 +999,39 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>27851</t>
+          <t>29141</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
+          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1041,39 +1041,39 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>27461</t>
+          <t>27851</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>법제처, 제3회 특별성과 포상 수여</t>
+          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1083,39 +1083,39 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>25671</t>
+          <t>27461</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
+          <t>법제처, 제3회 특별성과 포상 수여</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1125,39 +1125,39 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>24842</t>
+          <t>25671</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
+          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1167,29 +1167,29 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>24841</t>
+          <t>24842</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
+          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1221,27 +1221,27 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>23411</t>
+          <t>24841</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
+          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1251,34 +1251,34 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>23231</t>
+          <t>23411</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
+          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>법제자문1담당관</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1293,39 +1293,39 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>14381</t>
+          <t>23231</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
+          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>법제자문1담당관</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1335,39 +1335,39 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>14121</t>
+          <t>14381</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>법제로 완성하는 국가대전환</t>
+          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1377,39 +1377,39 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12952</t>
+          <t>14121</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
+          <t>법제로 완성하는 국가대전환</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1419,29 +1419,29 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12951</t>
+          <t>12952</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
+          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1473,27 +1473,27 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>11761</t>
+          <t>12951</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
+          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>법제교육과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1503,34 +1503,34 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>11711</t>
+          <t>11761</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
+          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법제교육과</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1545,39 +1545,39 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>11311</t>
+          <t>11711</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>범정부 형벌 합리화 추진단 공식 출범</t>
+          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>파견</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1587,39 +1587,39 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>4471</t>
+          <t>11311</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
+          <t>범정부 형벌 합리화 추진단 공식 출범</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>파견</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1629,39 +1629,39 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1511</t>
+          <t>4471</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
+          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1671,39 +1671,39 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>491</t>
+          <t>1511</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
+          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1713,39 +1713,39 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>491</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
+          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1755,29 +1755,29 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
+          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1809,27 +1809,27 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
+          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1851,27 +1851,27 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
+          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1893,27 +1893,27 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
+          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1935,27 +1935,27 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
+          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1977,27 +1977,27 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
+          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2019,27 +2019,27 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
+          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2061,27 +2061,27 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2103,40 +2103,82 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>대변인실</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>자율주행 규제 합리화, 해외직구 안전 강화 등 국민보호 · 산업지원 새 법령 시행</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150819&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>대변인실</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="H42" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-10-21 11:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -10936,7 +10936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10984,12 +10984,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>36</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>외국인 실명확인 서비스 일시 중단 안내(2026.10.24 (토) 22:00 ~ 10.25.(일) 04:00)</t>
+          <t>개인정보 유출신고시스템 작업에 따른 서비스 일시 중단 및 대체 신고 방법 안내</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -10999,39 +10999,39 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>20927</t>
+          <t>20928</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20927</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20928</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-20 11:01:57.312740+09:00</t>
+          <t>2026-10-21 10:47:12.040330+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-20 11:01:57.312740+09:00</t>
+          <t>2026-10-21 10:47:12.040330+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>개인정보 유출신고시스템 작업에 따른 서비스 일시 중단 및 대체 신고 방법 안내</t>
+          <t>외국인 실명확인 서비스 일시 중단 안내(2026.10.24 (토) 22:00 ~ 10.25.(일) 04:00)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11041,39 +11041,39 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>20924</t>
+          <t>20927</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20924</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20927</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-13 13:31:56.172770+09:00</t>
+          <t>2026-10-20 11:01:57.312740+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-13 13:31:56.172770+09:00</t>
+          <t>2026-10-20 11:01:57.312740+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>외국인 실명확인 서비스 일시 중단 안내(2026.10.8 (목) 18:00 ~ 10.9.(금) 11:00)</t>
+          <t>개인정보 유출신고시스템 작업에 따른 서비스 일시 중단 및 대체 신고 방법 안내</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -11083,39 +11083,39 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>20922</t>
+          <t>20924</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20922</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20924</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-09-28 15:01:57.296841+09:00</t>
+          <t>2026-10-13 13:31:56.172770+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-09-28 15:01:57.296841+09:00</t>
+          <t>2026-10-13 13:31:56.172770+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.10.18 (일) 00:00 ~10:00)</t>
+          <t>외국인 실명확인 서비스 일시 중단 안내(2026.10.8 (목) 18:00 ~ 10.9.(금) 11:00)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -11125,39 +11125,39 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>20921</t>
+          <t>20922</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20921</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20922</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-21 14:16:53.533733+09:00</t>
+          <t>2026-09-28 15:01:57.296841+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-21 14:16:53.533733+09:00</t>
+          <t>2026-09-28 15:01:57.296841+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>제6회 개인정보 보호의 날(9.30.) 기념식 개최</t>
+          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.10.18 (일) 00:00 ~10:00)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -11167,39 +11167,39 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>20920</t>
+          <t>20921</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20920</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20921</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-19 14:16:49.840552+09:00</t>
+          <t>2026-09-21 14:16:53.533733+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-19 14:16:49.840552+09:00</t>
+          <t>2026-09-21 14:16:53.533733+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026년 개인정보 보호주간(9.28.~10.2.) 포스터 및 앰블럼</t>
+          <t>제6회 개인정보 보호의 날(9.30.) 기념식 개최</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -11209,39 +11209,39 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>20917</t>
+          <t>20920</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20917</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20920</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-08 11:31:39.797854+09:00</t>
+          <t>2026-09-19 14:16:49.840552+09:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-08 11:31:39.797854+09:00</t>
+          <t>2026-09-19 14:16:49.840552+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 인증시험(2차) 안내</t>
+          <t>2026년 개인정보 보호주간(9.28.~10.2.) 포스터 및 앰블럼</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -11251,39 +11251,39 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>20915</t>
+          <t>20917</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20915</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20917</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-09-03 14:16:40.776731+09:00</t>
+          <t>2026-09-08 11:31:39.797854+09:00</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-03 14:16:40.776731+09:00</t>
+          <t>2026-09-08 11:31:39.797854+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>개인정보 포털 예방점검에 따른 서비스 중단 안내 (8.13 19:00 ~ 23:00)</t>
+          <t>2026년 개인정보 영향평가 인증시험(2차) 안내</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -11293,39 +11293,39 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>20909</t>
+          <t>20915</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20909</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20915</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-08-10 18:01:43.365104+09:00</t>
+          <t>2026-09-03 14:16:40.776731+09:00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-08-10 18:01:43.365104+09:00</t>
+          <t>2026-09-03 14:16:40.776731+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SKT  휴대폰 본인확인서비스 중단 공지(7.12 01:00 ~ 04:00)</t>
+          <t>개인정보 포털 예방점검에 따른 서비스 중단 안내 (8.13 19:00 ~ 23:00)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -11335,39 +11335,39 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>20908</t>
+          <t>20909</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20908</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20909</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-07-09 10:02:18.348370+09:00</t>
+          <t>2026-08-10 18:01:43.365104+09:00</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-07-09 10:02:18.348370+09:00</t>
+          <t>2026-08-10 18:01:43.365104+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 전문교육(하반기) 안내</t>
+          <t>SKT  휴대폰 본인확인서비스 중단 공지(7.12 01:00 ~ 04:00)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -11377,39 +11377,39 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>20907</t>
+          <t>20908</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20907</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20908</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-07-02 13:16:19.799934+09:00</t>
+          <t>2026-07-09 10:02:18.348370+09:00</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-02 13:16:19.799934+09:00</t>
+          <t>2026-07-09 10:02:18.348370+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.6.16 (화) 19:00 ~20:00)</t>
+          <t>2026년 개인정보 영향평가 전문교육(하반기) 안내</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -11419,17 +11419,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>20906</t>
+          <t>20907</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20906</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20907</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -11446,12 +11446,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
+          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.6.16 (화) 19:00 ~20:00)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -11461,17 +11461,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>20903</t>
+          <t>20906</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20903</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20906</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -11488,12 +11488,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>개인정보 포털 DB점검에 따른 서비스 중단 안내 (5.26 19:00 ~ 21:00)</t>
+          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -11503,17 +11503,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>20900</t>
+          <t>20903</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20900</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20903</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -11530,12 +11530,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>(복구완료) 외국인 실명확인 서비스 장애 안내(26.05.19 13:47 ~18:50 )</t>
+          <t>개인정보 포털 DB점검에 따른 서비스 중단 안내 (5.26 19:00 ~ 21:00)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -11545,17 +11545,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>20896</t>
+          <t>20900</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20896</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20900</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -11572,12 +11572,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>제3기 가명정보 전문가 풀 모집 공고</t>
+          <t>(복구완료) 외국인 실명확인 서비스 장애 안내(26.05.19 13:47 ~18:50 )</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -11587,17 +11587,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>20895</t>
+          <t>20896</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20895</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20896</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -11614,12 +11614,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>SKT 휴대폰 본인확인서비스 중단 공지(5.10 03:20 ~ 03:25 / 5.12 03:20 ~ 03:25)</t>
+          <t>제3기 가명정보 전문가 풀 모집 공고</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -11629,17 +11629,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>20894</t>
+          <t>20895</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20894</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20895</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -11656,12 +11656,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 인증시험(1차) 안내</t>
+          <t>SKT 휴대폰 본인확인서비스 중단 공지(5.10 03:20 ~ 03:25 / 5.12 03:20 ~ 03:25)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -11671,17 +11671,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>20893</t>
+          <t>20894</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20893</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20894</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -11698,12 +11698,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>본인인증 서비스 장애 발생 공지(2026.04.28(화)15:00 ~ 15:10)</t>
+          <t>2026년 개인정보 영향평가 인증시험(1차) 안내</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -11713,17 +11713,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>20888</t>
+          <t>20893</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20888</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20893</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -11740,12 +11740,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>개인정보 영향평가 전문인력 인증서 발급 및 유효기간 관련 안내</t>
+          <t>본인인증 서비스 장애 발생 공지(2026.04.28(화)15:00 ~ 15:10)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -11755,17 +11755,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>20884</t>
+          <t>20888</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20884</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20888</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -11782,12 +11782,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 계속교육 일정 안내</t>
+          <t>개인정보 영향평가 전문인력 인증서 발급 및 유효기간 관련 안내</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -11797,17 +11797,17 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>20878</t>
+          <t>20884</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20878</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20884</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -11824,12 +11824,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.4.8 (수) 03:00 ~05:00)</t>
+          <t>2026년 개인정보 영향평가 계속교육 일정 안내</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -11839,17 +11839,17 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>20875</t>
+          <t>20878</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20875</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20878</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -11866,12 +11866,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내 (2026년 3월 24일(화) 23:00~ 3월 25일(수) 02:00)</t>
+          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.4.8 (수) 03:00 ~05:00)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -11881,17 +11881,17 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>20874</t>
+          <t>20875</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20874</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20875</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -11908,12 +11908,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.03.24(화)22:00 ~ 2026.03.25(수) 02:00)</t>
+          <t>본인확인 서비스 작업 공지 안내 (2026년 3월 24일(화) 23:00~ 3월 25일(수) 02:00)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -11928,12 +11928,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>20873</t>
+          <t>20874</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20873</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20874</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -11950,12 +11950,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 전문교육(상반기) 안내</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.03.24(화)22:00 ~ 2026.03.25(수) 02:00)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -11970,12 +11970,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>20872</t>
+          <t>20873</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20872</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20873</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -11992,12 +11992,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>외국인 실명확인 서비스 작업 공지 안내</t>
+          <t>2026년 개인정보 영향평가 전문교육(상반기) 안내</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -12007,17 +12007,17 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>20871</t>
+          <t>20872</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20871</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20872</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -12034,12 +12034,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.03.24. (화) 02:00 ~ 04:00)</t>
+          <t>외국인 실명확인 서비스 작업 공지 안내</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -12049,17 +12049,17 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>20870</t>
+          <t>20871</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20870</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20871</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -12076,12 +12076,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.01.22 (목) 22:00 ~2026.01.23 (금) 05:00)</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.03.24. (화) 02:00 ~ 04:00)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -12091,17 +12091,17 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>20868</t>
+          <t>20870</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20868</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20870</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -12118,12 +12118,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.01.21 (수) 19:00 ~21:00)</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.01.22 (목) 22:00 ~2026.01.23 (금) 05:00)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -12133,17 +12133,17 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>20867</t>
+          <t>20868</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20867</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20868</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -12160,12 +12160,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>개인정보 포털 사용자 편의성 설문조사 참여 이벤트 당첨자 발표</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.01.21 (수) 19:00 ~21:00)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -12175,17 +12175,17 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>20866</t>
+          <t>20867</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20866</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20867</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -12202,12 +12202,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 보호·활용 분야 R&amp;amp;D 사업 신규지원 대상과제 공고(~2.10. 오후 3시)</t>
+          <t>개인정보 포털 사용자 편의성 설문조사 참여 이벤트 당첨자 발표</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -12217,17 +12217,17 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>20865</t>
+          <t>20866</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20865</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20866</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -12244,12 +12244,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.1.12 (월) 05:00 ~06:00)</t>
+          <t>2026년도 개인정보 보호·활용 분야 R&amp;amp;D 사업 신규지원 대상과제 공고(~2.10. 오후 3시)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -12259,17 +12259,17 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>20862</t>
+          <t>20865</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20862</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20865</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -12286,12 +12286,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>「개인정보관리 전문기관 지정 심사위원회」 심사위원 모집 안내 (~12.23. 18시까지)</t>
+          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.1.12 (월) 05:00 ~06:00)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -12301,17 +12301,17 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>20856</t>
+          <t>20862</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20856</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20862</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -12328,12 +12328,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>외국인 본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.17 (수) 16:00 ~17:00)</t>
+          <t>「개인정보관리 전문기관 지정 심사위원회」 심사위원 모집 안내 (~12.23. 18시까지)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -12343,17 +12343,17 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>20855</t>
+          <t>20856</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20855</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20856</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -12370,12 +12370,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.15 (월) 08:00 ~09:00)</t>
+          <t>외국인 본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.17 (수) 16:00 ~17:00)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -12390,12 +12390,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>20854</t>
+          <t>20855</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20854</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20855</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -12412,40 +12412,82 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.15 (월) 08:00 ~09:00)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>관리자</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>20854</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20854</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:16:19.799934+09:00</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:16:19.799934+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>2025년 개인정보 영향평가 인증시험(2차) 안내</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>관리자</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>2025-08-25</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>20837</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20837</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>2026-07-02 13:16:19.799934+09:00</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="H37" t="inlineStr">
         <is>
           <t>2026-07-02 13:16:19.799934+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-10-21 17:20:02 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,27 +465,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>45121</t>
+          <t>45631</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>국민의 생애주기에 맞춘 생활법령정보 서비스 발전 방안 논의</t>
+          <t>“법을 얼마나 알고 있나요?” 법제처, 청소년 골든벨 대회 개최</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158862&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158921&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -495,39 +495,39 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-20 14:45:19.906187+09:00</t>
+          <t>2026-10-21 17:15:20.296716+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-20 14:45:19.906187+09:00</t>
+          <t>2026-10-21 17:15:20.296716+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>41651</t>
+          <t>45121</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>법제처, 지방정부 등의 자치법규 입안을 위한 종합안내서 발간</t>
+          <t>국민의 생애주기에 맞춘 생활법령정보 서비스 발전 방안 논의</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158475&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158862&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -537,39 +537,39 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-12 10:00:18.987080+09:00</t>
+          <t>2026-10-20 14:45:19.906187+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-12 10:00:18.987080+09:00</t>
+          <t>2026-10-20 14:45:19.906187+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>37711</t>
+          <t>41651</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>“행정기본법 제정 5주년, 새로운 길을 찾다”</t>
+          <t>법제처, 지방정부 등의 자치법규 입안을 위한 종합안내서 발간</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157976&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158475&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -579,34 +579,34 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-02 14:00:20.071730+09:00</t>
+          <t>2026-10-12 10:00:18.987080+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-10-02 14:00:20.071730+09:00</t>
+          <t>2026-10-12 10:00:18.987080+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>37581</t>
+          <t>37711</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>국민이 직접 뽑은 ‘대표 알기 쉬운 법령 용어’에 “사위(詐僞) → 거짓/속임수” 등 5개 선정</t>
+          <t>“행정기본법 제정 5주년, 새로운 길을 찾다”</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157972&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157976&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -621,29 +621,29 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-02 10:45:20.519914+09:00</t>
+          <t>2026-10-02 14:00:20.071730+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-02 10:45:20.519914+09:00</t>
+          <t>2026-10-02 14:00:20.071730+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>37351</t>
+          <t>37581</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>법제처, 알기 쉬운 법령 만들기 20년을 돌아보고 미래를 이야기하다!</t>
+          <t>국민이 직접 뽑은 ‘대표 알기 쉬운 법령 용어’에 “사위(詐僞) → 거짓/속임수” 등 5개 선정</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157915&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157972&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -653,7 +653,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -663,34 +663,34 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-01 15:15:21.104965+09:00</t>
+          <t>2026-10-02 10:45:20.519914+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-01 15:15:21.104965+09:00</t>
+          <t>2026-10-02 10:45:20.519914+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>37152</t>
+          <t>37351</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>가상자산 활용 보이스피싱 피해 구제 확대 및 배달앱 원산지 표시 고지 의무화</t>
+          <t>법제처, 알기 쉬운 법령 만들기 20년을 돌아보고 미래를 이야기하다!</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157902&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157915&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -705,29 +705,29 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-01 10:15:19.890918+09:00</t>
+          <t>2026-10-01 15:15:21.104965+09:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-01 10:15:19.890918+09:00</t>
+          <t>2026-10-01 15:15:21.104965+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>37151</t>
+          <t>37152</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Expanding Voice Phishing Damage Relief Utilizing Virtual Assets and ..</t>
+          <t>가상자산 활용 보이스피싱 피해 구제 확대 및 배달앱 원산지 표시 고지 의무화</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157904&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157902&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -759,17 +759,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>36341</t>
+          <t>37151</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>법제처, AI로 국민과 법의 거리를 좁힌다</t>
+          <t>Expanding Voice Phishing Damage Relief Utilizing Virtual Assets and ..</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157747&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157904&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -789,39 +789,39 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-09-29 10:30:21.085354+09:00</t>
+          <t>2026-10-01 10:15:19.890918+09:00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-29 10:30:21.085354+09:00</t>
+          <t>2026-10-01 10:15:19.890918+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>33671</t>
+          <t>36341</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
+          <t>법제처, AI로 국민과 법의 거리를 좁힌다</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157747&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>법제조정법제관실</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -831,39 +831,39 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-09-22 15:30:19.394844+09:00</t>
+          <t>2026-09-29 10:30:21.085354+09:00</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-22 15:30:19.394844+09:00</t>
+          <t>2026-09-29 10:30:21.085354+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>33082</t>
+          <t>33671</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
+          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>법제조정법제관실</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -873,29 +873,29 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>31861</t>
+          <t>33082</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
+          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -915,39 +915,39 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>31651</t>
+          <t>31861</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
+          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>경제법제국</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -957,39 +957,39 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>31201</t>
+          <t>31651</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
+          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>경제법제국</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -999,29 +999,29 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>29141</t>
+          <t>31201</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
+          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1041,39 +1041,39 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>27851</t>
+          <t>29141</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
+          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1083,39 +1083,39 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>27461</t>
+          <t>27851</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>법제처, 제3회 특별성과 포상 수여</t>
+          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1125,39 +1125,39 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>25671</t>
+          <t>27461</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
+          <t>법제처, 제3회 특별성과 포상 수여</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1167,39 +1167,39 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>24842</t>
+          <t>25671</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
+          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1209,29 +1209,29 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>24841</t>
+          <t>24842</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
+          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1263,27 +1263,27 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>23411</t>
+          <t>24841</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
+          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1293,34 +1293,34 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>23231</t>
+          <t>23411</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
+          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>법제자문1담당관</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1335,39 +1335,39 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>14381</t>
+          <t>23231</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
+          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>법제자문1담당관</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1377,39 +1377,39 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>14121</t>
+          <t>14381</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>법제로 완성하는 국가대전환</t>
+          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1419,39 +1419,39 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12952</t>
+          <t>14121</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
+          <t>법제로 완성하는 국가대전환</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1461,29 +1461,29 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12951</t>
+          <t>12952</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
+          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1515,27 +1515,27 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>11761</t>
+          <t>12951</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
+          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>법제교육과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1545,34 +1545,34 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>11711</t>
+          <t>11761</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
+          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법제교육과</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1587,39 +1587,39 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>11311</t>
+          <t>11711</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>범정부 형벌 합리화 추진단 공식 출범</t>
+          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>파견</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1629,39 +1629,39 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>4471</t>
+          <t>11311</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
+          <t>범정부 형벌 합리화 추진단 공식 출범</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>파견</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1671,39 +1671,39 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1511</t>
+          <t>4471</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
+          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1713,39 +1713,39 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>491</t>
+          <t>1511</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
+          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1755,39 +1755,39 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>491</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
+          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1797,29 +1797,29 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
+          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1851,27 +1851,27 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
+          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1893,27 +1893,27 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
+          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1935,27 +1935,27 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
+          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1977,27 +1977,27 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
+          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2019,27 +2019,27 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
+          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2061,27 +2061,27 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
+          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2103,27 +2103,27 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2145,40 +2145,82 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>대변인실</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>자율주행 규제 합리화, 해외직구 안전 강화 등 국민보호 · 산업지원 새 법령 시행</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150819&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>대변인실</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-10-26 14:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -11149,7 +11149,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11197,12 +11197,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>37</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>개인정보 유출신고시스템 작업에 따른 서비스 일시 중단 및 대체 신고 방법 안내</t>
+          <t>개인정보 유출신고시스템 작업에 따른 서비스 일시 중단 및 대체 신고 방법 안내(10.27.(화) 18:00 ~ 10.28.(수) 08:00)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -11212,39 +11212,39 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>20928</t>
+          <t>20930</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20928</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20930</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-21 10:47:12.040330+09:00</t>
+          <t>2026-10-26 14:01:53.055892+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-21 10:47:12.040330+09:00</t>
+          <t>2026-10-26 14:01:53.055892+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>36</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>외국인 실명확인 서비스 일시 중단 안내(2026.10.24 (토) 22:00 ~ 10.25.(일) 04:00)</t>
+          <t>개인정보 유출신고시스템 작업에 따른 서비스 일시 중단 및 대체 신고 방법 안내</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11254,39 +11254,39 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>20927</t>
+          <t>20928</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20927</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20928</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-20 11:01:57.312740+09:00</t>
+          <t>2026-10-21 10:47:12.040330+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-20 11:01:57.312740+09:00</t>
+          <t>2026-10-21 10:47:12.040330+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>개인정보 유출신고시스템 작업에 따른 서비스 일시 중단 및 대체 신고 방법 안내</t>
+          <t>외국인 실명확인 서비스 일시 중단 안내(2026.10.24 (토) 22:00 ~ 10.25.(일) 04:00)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -11296,39 +11296,39 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>20924</t>
+          <t>20927</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20924</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20927</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-13 13:31:56.172770+09:00</t>
+          <t>2026-10-20 11:01:57.312740+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-10-13 13:31:56.172770+09:00</t>
+          <t>2026-10-20 11:01:57.312740+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>외국인 실명확인 서비스 일시 중단 안내(2026.10.8 (목) 18:00 ~ 10.9.(금) 11:00)</t>
+          <t>개인정보 유출신고시스템 작업에 따른 서비스 일시 중단 및 대체 신고 방법 안내</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -11338,39 +11338,39 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>20922</t>
+          <t>20924</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20922</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20924</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-28 15:01:57.296841+09:00</t>
+          <t>2026-10-13 13:31:56.172770+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-28 15:01:57.296841+09:00</t>
+          <t>2026-10-13 13:31:56.172770+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.10.18 (일) 00:00 ~10:00)</t>
+          <t>외국인 실명확인 서비스 일시 중단 안내(2026.10.8 (목) 18:00 ~ 10.9.(금) 11:00)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -11380,39 +11380,39 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>20921</t>
+          <t>20922</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20921</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20922</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-21 14:16:53.533733+09:00</t>
+          <t>2026-09-28 15:01:57.296841+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-21 14:16:53.533733+09:00</t>
+          <t>2026-09-28 15:01:57.296841+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>제6회 개인정보 보호의 날(9.30.) 기념식 개최</t>
+          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.10.18 (일) 00:00 ~10:00)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -11422,39 +11422,39 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>20920</t>
+          <t>20921</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20920</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20921</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-19 14:16:49.840552+09:00</t>
+          <t>2026-09-21 14:16:53.533733+09:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-19 14:16:49.840552+09:00</t>
+          <t>2026-09-21 14:16:53.533733+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026년 개인정보 보호주간(9.28.~10.2.) 포스터 및 앰블럼</t>
+          <t>제6회 개인정보 보호의 날(9.30.) 기념식 개최</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -11464,39 +11464,39 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>20917</t>
+          <t>20920</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20917</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20920</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-09-08 11:31:39.797854+09:00</t>
+          <t>2026-09-19 14:16:49.840552+09:00</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-08 11:31:39.797854+09:00</t>
+          <t>2026-09-19 14:16:49.840552+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 인증시험(2차) 안내</t>
+          <t>2026년 개인정보 보호주간(9.28.~10.2.) 포스터 및 앰블럼</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -11506,39 +11506,39 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>20915</t>
+          <t>20917</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20915</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20917</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-09-03 14:16:40.776731+09:00</t>
+          <t>2026-09-08 11:31:39.797854+09:00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-03 14:16:40.776731+09:00</t>
+          <t>2026-09-08 11:31:39.797854+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>개인정보 포털 예방점검에 따른 서비스 중단 안내 (8.13 19:00 ~ 23:00)</t>
+          <t>2026년 개인정보 영향평가 인증시험(2차) 안내</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -11548,39 +11548,39 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>20909</t>
+          <t>20915</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20909</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20915</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-08-10 18:01:43.365104+09:00</t>
+          <t>2026-09-03 14:16:40.776731+09:00</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-10 18:01:43.365104+09:00</t>
+          <t>2026-09-03 14:16:40.776731+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>SKT  휴대폰 본인확인서비스 중단 공지(7.12 01:00 ~ 04:00)</t>
+          <t>개인정보 포털 예방점검에 따른 서비스 중단 안내 (8.13 19:00 ~ 23:00)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -11590,39 +11590,39 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>20908</t>
+          <t>20909</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20908</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20909</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-07-09 10:02:18.348370+09:00</t>
+          <t>2026-08-10 18:01:43.365104+09:00</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-09 10:02:18.348370+09:00</t>
+          <t>2026-08-10 18:01:43.365104+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 전문교육(하반기) 안내</t>
+          <t>SKT  휴대폰 본인확인서비스 중단 공지(7.12 01:00 ~ 04:00)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -11632,39 +11632,39 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>20907</t>
+          <t>20908</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20907</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20908</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-07-02 13:16:19.799934+09:00</t>
+          <t>2026-07-09 10:02:18.348370+09:00</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-07-02 13:16:19.799934+09:00</t>
+          <t>2026-07-09 10:02:18.348370+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.6.16 (화) 19:00 ~20:00)</t>
+          <t>2026년 개인정보 영향평가 전문교육(하반기) 안내</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -11674,17 +11674,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>20906</t>
+          <t>20907</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20906</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20907</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -11701,12 +11701,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
+          <t>정보주체 권리행사(본인확인 내역조회, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.6.16 (화) 19:00 ~20:00)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -11716,17 +11716,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>20903</t>
+          <t>20906</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20903</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20906</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -11743,12 +11743,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>개인정보 포털 DB점검에 따른 서비스 중단 안내 (5.26 19:00 ~ 21:00)</t>
+          <t>개인정보보호 중심 설계(PbD) 시범인증 참여제품 모집 공고</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -11758,17 +11758,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>20900</t>
+          <t>20903</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20900</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20903</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -11785,12 +11785,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>(복구완료) 외국인 실명확인 서비스 장애 안내(26.05.19 13:47 ~18:50 )</t>
+          <t>개인정보 포털 DB점검에 따른 서비스 중단 안내 (5.26 19:00 ~ 21:00)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -11800,17 +11800,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>20896</t>
+          <t>20900</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20896</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20900</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -11827,12 +11827,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>제3기 가명정보 전문가 풀 모집 공고</t>
+          <t>(복구완료) 외국인 실명확인 서비스 장애 안내(26.05.19 13:47 ~18:50 )</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -11842,17 +11842,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>20895</t>
+          <t>20896</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20895</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20896</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -11869,12 +11869,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>SKT 휴대폰 본인확인서비스 중단 공지(5.10 03:20 ~ 03:25 / 5.12 03:20 ~ 03:25)</t>
+          <t>제3기 가명정보 전문가 풀 모집 공고</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -11884,17 +11884,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>20894</t>
+          <t>20895</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20894</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20895</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -11911,12 +11911,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 인증시험(1차) 안내</t>
+          <t>SKT 휴대폰 본인확인서비스 중단 공지(5.10 03:20 ~ 03:25 / 5.12 03:20 ~ 03:25)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -11926,17 +11926,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>20893</t>
+          <t>20894</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20893</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20894</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -11953,12 +11953,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>본인인증 서비스 장애 발생 공지(2026.04.28(화)15:00 ~ 15:10)</t>
+          <t>2026년 개인정보 영향평가 인증시험(1차) 안내</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -11968,17 +11968,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>20888</t>
+          <t>20893</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20888</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20893</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -11995,12 +11995,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>개인정보 영향평가 전문인력 인증서 발급 및 유효기간 관련 안내</t>
+          <t>본인인증 서비스 장애 발생 공지(2026.04.28(화)15:00 ~ 15:10)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -12010,17 +12010,17 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>20884</t>
+          <t>20888</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20884</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20888</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -12037,12 +12037,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 계속교육 일정 안내</t>
+          <t>개인정보 영향평가 전문인력 인증서 발급 및 유효기간 관련 안내</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -12052,17 +12052,17 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>20878</t>
+          <t>20884</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20878</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20884</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -12079,12 +12079,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.4.8 (수) 03:00 ~05:00)</t>
+          <t>2026년 개인정보 영향평가 계속교육 일정 안내</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -12094,17 +12094,17 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>20875</t>
+          <t>20878</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20875</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20878</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -12121,12 +12121,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내 (2026년 3월 24일(화) 23:00~ 3월 25일(수) 02:00)</t>
+          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.4.8 (수) 03:00 ~05:00)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -12136,17 +12136,17 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>20874</t>
+          <t>20875</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20874</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20875</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -12163,12 +12163,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.03.24(화)22:00 ~ 2026.03.25(수) 02:00)</t>
+          <t>본인확인 서비스 작업 공지 안내 (2026년 3월 24일(화) 23:00~ 3월 25일(수) 02:00)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -12183,12 +12183,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>20873</t>
+          <t>20874</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20873</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20874</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -12205,12 +12205,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026년 개인정보 영향평가 전문교육(상반기) 안내</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.03.24(화)22:00 ~ 2026.03.25(수) 02:00)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -12225,12 +12225,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>20872</t>
+          <t>20873</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20872</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20873</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -12247,12 +12247,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>외국인 실명확인 서비스 작업 공지 안내</t>
+          <t>2026년 개인정보 영향평가 전문교육(상반기) 안내</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -12262,17 +12262,17 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>20871</t>
+          <t>20872</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20871</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20872</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -12289,12 +12289,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.03.24. (화) 02:00 ~ 04:00)</t>
+          <t>외국인 실명확인 서비스 작업 공지 안내</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -12304,17 +12304,17 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>20870</t>
+          <t>20871</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20870</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20871</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -12331,12 +12331,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.01.22 (목) 22:00 ~2026.01.23 (금) 05:00)</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.03.24. (화) 02:00 ~ 04:00)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -12346,17 +12346,17 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>20868</t>
+          <t>20870</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20868</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20870</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -12373,12 +12373,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>본인확인 서비스 작업 공지 안내(2026.01.21 (수) 19:00 ~21:00)</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.01.22 (목) 22:00 ~2026.01.23 (금) 05:00)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -12388,17 +12388,17 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>20867</t>
+          <t>20868</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20867</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20868</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -12415,12 +12415,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>개인정보 포털 사용자 편의성 설문조사 참여 이벤트 당첨자 발표</t>
+          <t>본인확인 서비스 작업 공지 안내(2026.01.21 (수) 19:00 ~21:00)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -12430,17 +12430,17 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>20866</t>
+          <t>20867</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20866</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20867</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -12457,12 +12457,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026년도 개인정보 보호·활용 분야 R&amp;amp;D 사업 신규지원 대상과제 공고(~2.10. 오후 3시)</t>
+          <t>개인정보 포털 사용자 편의성 설문조사 참여 이벤트 당첨자 발표</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -12472,17 +12472,17 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>20865</t>
+          <t>20866</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20865</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20866</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -12499,12 +12499,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.1.12 (월) 05:00 ~06:00)</t>
+          <t>2026년도 개인정보 보호·활용 분야 R&amp;amp;D 사업 신규지원 대상과제 공고(~2.10. 오후 3시)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -12514,17 +12514,17 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>20862</t>
+          <t>20865</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20862</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20865</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -12541,12 +12541,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>「개인정보관리 전문기관 지정 심사위원회」 심사위원 모집 안내 (~12.23. 18시까지)</t>
+          <t>정보주체 권리행사(본인인증 내역확인, 웹사이트 회원탈퇴) 서비스 일시 중단 안내 (2026.1.12 (월) 05:00 ~06:00)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -12556,17 +12556,17 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>20856</t>
+          <t>20862</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20856</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20862</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -12583,12 +12583,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>외국인 본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.17 (수) 16:00 ~17:00)</t>
+          <t>「개인정보관리 전문기관 지정 심사위원회」 심사위원 모집 안내 (~12.23. 18시까지)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -12598,17 +12598,17 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>20855</t>
+          <t>20856</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20855</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20856</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -12625,12 +12625,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.15 (월) 08:00 ~09:00)</t>
+          <t>외국인 본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.17 (수) 16:00 ~17:00)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -12645,12 +12645,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>20854</t>
+          <t>20855</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20854</t>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20855</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -12667,40 +12667,82 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>본인확인/아이핀/실명확인 서비스 일시 중단 안내(2025.12.15 (월) 08:00 ~09:00)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>관리자</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>20854</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20854</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:16:19.799934+09:00</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:16:19.799934+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>2025년 개인정보 영향평가 인증시험(2차) 안내</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>관리자</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>2025-08-25</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>20837</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>https://www.privacy.go.kr/front/bbs/bbsView.do?bbsNo=BBSMSTR_000000000001&amp;bbscttNo=20837</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>2026-07-02 13:16:19.799934+09:00</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>2026-07-02 13:16:19.799934+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-10-27 14:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,27 +465,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>45631</t>
+          <t>47941</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>“법을 얼마나 알고 있나요?” 법제처, 청소년 골든벨 대회 개최</t>
+          <t>실무경력 인정 범위를 넓혀, 청년의 사회진출 돕는다</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158921&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=159220&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법령품질개선과</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -495,39 +495,39 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-21 17:15:20.296716+09:00</t>
+          <t>2026-10-27 13:30:19.056395+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-21 17:15:20.296716+09:00</t>
+          <t>2026-10-27 13:30:19.056395+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>45121</t>
+          <t>45631</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>국민의 생애주기에 맞춘 생활법령정보 서비스 발전 방안 논의</t>
+          <t>“법을 얼마나 알고 있나요?” 법제처, 청소년 골든벨 대회 개최</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158862&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158921&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -537,39 +537,39 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-20 14:45:19.906187+09:00</t>
+          <t>2026-10-21 17:15:20.296716+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-20 14:45:19.906187+09:00</t>
+          <t>2026-10-21 17:15:20.296716+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>41651</t>
+          <t>45121</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>법제처, 지방정부 등의 자치법규 입안을 위한 종합안내서 발간</t>
+          <t>국민의 생애주기에 맞춘 생활법령정보 서비스 발전 방안 논의</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158475&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158862&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -579,39 +579,39 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-12 10:00:18.987080+09:00</t>
+          <t>2026-10-20 14:45:19.906187+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-10-12 10:00:18.987080+09:00</t>
+          <t>2026-10-20 14:45:19.906187+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>37711</t>
+          <t>41651</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>“행정기본법 제정 5주년, 새로운 길을 찾다”</t>
+          <t>법제처, 지방정부 등의 자치법규 입안을 위한 종합안내서 발간</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157976&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158475&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -621,34 +621,34 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-02 14:00:20.071730+09:00</t>
+          <t>2026-10-12 10:00:18.987080+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-02 14:00:20.071730+09:00</t>
+          <t>2026-10-12 10:00:18.987080+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>37581</t>
+          <t>37711</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>국민이 직접 뽑은 ‘대표 알기 쉬운 법령 용어’에 “사위(詐僞) → 거짓/속임수” 등 5개 선정</t>
+          <t>“행정기본법 제정 5주년, 새로운 길을 찾다”</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157972&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157976&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -663,29 +663,29 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-02 10:45:20.519914+09:00</t>
+          <t>2026-10-02 14:00:20.071730+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-02 10:45:20.519914+09:00</t>
+          <t>2026-10-02 14:00:20.071730+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>37351</t>
+          <t>37581</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>법제처, 알기 쉬운 법령 만들기 20년을 돌아보고 미래를 이야기하다!</t>
+          <t>국민이 직접 뽑은 ‘대표 알기 쉬운 법령 용어’에 “사위(詐僞) → 거짓/속임수” 등 5개 선정</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157915&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157972&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -705,34 +705,34 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-01 15:15:21.104965+09:00</t>
+          <t>2026-10-02 10:45:20.519914+09:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-01 15:15:21.104965+09:00</t>
+          <t>2026-10-02 10:45:20.519914+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>37152</t>
+          <t>37351</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>가상자산 활용 보이스피싱 피해 구제 확대 및 배달앱 원산지 표시 고지 의무화</t>
+          <t>법제처, 알기 쉬운 법령 만들기 20년을 돌아보고 미래를 이야기하다!</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157902&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157915&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -747,29 +747,29 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-01 10:15:19.890918+09:00</t>
+          <t>2026-10-01 15:15:21.104965+09:00</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-01 10:15:19.890918+09:00</t>
+          <t>2026-10-01 15:15:21.104965+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>37151</t>
+          <t>37152</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Expanding Voice Phishing Damage Relief Utilizing Virtual Assets and ..</t>
+          <t>가상자산 활용 보이스피싱 피해 구제 확대 및 배달앱 원산지 표시 고지 의무화</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157904&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157902&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -801,17 +801,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>36341</t>
+          <t>37151</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>법제처, AI로 국민과 법의 거리를 좁힌다</t>
+          <t>Expanding Voice Phishing Damage Relief Utilizing Virtual Assets and ..</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157747&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157904&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -831,39 +831,39 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-09-29 10:30:21.085354+09:00</t>
+          <t>2026-10-01 10:15:19.890918+09:00</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-29 10:30:21.085354+09:00</t>
+          <t>2026-10-01 10:15:19.890918+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>33671</t>
+          <t>36341</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
+          <t>법제처, AI로 국민과 법의 거리를 좁힌다</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157747&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>법제조정법제관실</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -873,39 +873,39 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-09-22 15:30:19.394844+09:00</t>
+          <t>2026-09-29 10:30:21.085354+09:00</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-22 15:30:19.394844+09:00</t>
+          <t>2026-09-29 10:30:21.085354+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>33082</t>
+          <t>33671</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
+          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>법제조정법제관실</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -915,29 +915,29 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>31861</t>
+          <t>33082</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
+          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -957,39 +957,39 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>31651</t>
+          <t>31861</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
+          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>경제법제국</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -999,39 +999,39 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>31201</t>
+          <t>31651</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
+          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>경제법제국</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1041,29 +1041,29 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>29141</t>
+          <t>31201</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
+          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1083,39 +1083,39 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>27851</t>
+          <t>29141</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
+          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1125,39 +1125,39 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>27461</t>
+          <t>27851</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>법제처, 제3회 특별성과 포상 수여</t>
+          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1167,39 +1167,39 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>25671</t>
+          <t>27461</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
+          <t>법제처, 제3회 특별성과 포상 수여</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1209,39 +1209,39 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>24842</t>
+          <t>25671</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
+          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1251,29 +1251,29 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>24841</t>
+          <t>24842</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
+          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1305,27 +1305,27 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>23411</t>
+          <t>24841</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
+          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1335,34 +1335,34 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>23231</t>
+          <t>23411</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
+          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>법제자문1담당관</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1377,39 +1377,39 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>14381</t>
+          <t>23231</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
+          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>법제자문1담당관</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1419,39 +1419,39 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>14121</t>
+          <t>14381</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>법제로 완성하는 국가대전환</t>
+          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1461,39 +1461,39 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12952</t>
+          <t>14121</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
+          <t>법제로 완성하는 국가대전환</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1503,29 +1503,29 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>12951</t>
+          <t>12952</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
+          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1557,27 +1557,27 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>11761</t>
+          <t>12951</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
+          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>법제교육과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1587,34 +1587,34 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>11711</t>
+          <t>11761</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
+          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법제교육과</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1629,39 +1629,39 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>11311</t>
+          <t>11711</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>범정부 형벌 합리화 추진단 공식 출범</t>
+          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>파견</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1671,39 +1671,39 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>4471</t>
+          <t>11311</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
+          <t>범정부 형벌 합리화 추진단 공식 출범</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>파견</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1713,39 +1713,39 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1511</t>
+          <t>4471</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
+          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1755,39 +1755,39 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>491</t>
+          <t>1511</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
+          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1797,39 +1797,39 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>491</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
+          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1839,29 +1839,29 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
+          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1893,27 +1893,27 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
+          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1935,27 +1935,27 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
+          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1977,27 +1977,27 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
+          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2019,27 +2019,27 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
+          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2061,27 +2061,27 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
+          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2103,27 +2103,27 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
+          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2145,27 +2145,27 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2187,40 +2187,82 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>대변인실</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>자율주행 규제 합리화, 해외직구 안전 강화 등 국민보호 · 산업지원 새 법령 시행</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150819&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>대변인실</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="H44" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-10-29 10:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,27 +465,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>47941</t>
+          <t>48631</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>실무경력 인정 범위를 넓혀, 청년의 사회진출 돕는다</t>
+          <t>전통시장에서 찾는 일상 속 법 보물... K-법 생활발견 캠페인 ‘숨은 법 보물찾기’ 개최</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=159220&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=159333&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>법령품질개선과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -495,39 +495,39 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-27 13:30:19.056395+09:00</t>
+          <t>2026-10-29 10:15:19.676658+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-27 13:30:19.056395+09:00</t>
+          <t>2026-10-29 10:15:19.676658+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>45631</t>
+          <t>47941</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>“법을 얼마나 알고 있나요?” 법제처, 청소년 골든벨 대회 개최</t>
+          <t>실무경력 인정 범위를 넓혀, 청년의 사회진출 돕는다</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158921&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=159220&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법령품질개선과</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -537,39 +537,39 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-21 17:15:20.296716+09:00</t>
+          <t>2026-10-27 13:30:19.056395+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-21 17:15:20.296716+09:00</t>
+          <t>2026-10-27 13:30:19.056395+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>45121</t>
+          <t>45631</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>국민의 생애주기에 맞춘 생활법령정보 서비스 발전 방안 논의</t>
+          <t>“법을 얼마나 알고 있나요?” 법제처, 청소년 골든벨 대회 개최</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158862&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158921&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -579,39 +579,39 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-20 14:45:19.906187+09:00</t>
+          <t>2026-10-21 17:15:20.296716+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-10-20 14:45:19.906187+09:00</t>
+          <t>2026-10-21 17:15:20.296716+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>41651</t>
+          <t>45121</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>법제처, 지방정부 등의 자치법규 입안을 위한 종합안내서 발간</t>
+          <t>국민의 생애주기에 맞춘 생활법령정보 서비스 발전 방안 논의</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158475&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158862&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -621,39 +621,39 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-12 10:00:18.987080+09:00</t>
+          <t>2026-10-20 14:45:19.906187+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-12 10:00:18.987080+09:00</t>
+          <t>2026-10-20 14:45:19.906187+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>37711</t>
+          <t>41651</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>“행정기본법 제정 5주년, 새로운 길을 찾다”</t>
+          <t>법제처, 지방정부 등의 자치법규 입안을 위한 종합안내서 발간</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157976&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158475&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -663,34 +663,34 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-02 14:00:20.071730+09:00</t>
+          <t>2026-10-12 10:00:18.987080+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-02 14:00:20.071730+09:00</t>
+          <t>2026-10-12 10:00:18.987080+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>37581</t>
+          <t>37711</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>국민이 직접 뽑은 ‘대표 알기 쉬운 법령 용어’에 “사위(詐僞) → 거짓/속임수” 등 5개 선정</t>
+          <t>“행정기본법 제정 5주년, 새로운 길을 찾다”</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157972&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157976&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -705,29 +705,29 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-02 10:45:20.519914+09:00</t>
+          <t>2026-10-02 14:00:20.071730+09:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-02 10:45:20.519914+09:00</t>
+          <t>2026-10-02 14:00:20.071730+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>37351</t>
+          <t>37581</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>법제처, 알기 쉬운 법령 만들기 20년을 돌아보고 미래를 이야기하다!</t>
+          <t>국민이 직접 뽑은 ‘대표 알기 쉬운 법령 용어’에 “사위(詐僞) → 거짓/속임수” 등 5개 선정</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157915&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157972&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -737,7 +737,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -747,34 +747,34 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-01 15:15:21.104965+09:00</t>
+          <t>2026-10-02 10:45:20.519914+09:00</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-01 15:15:21.104965+09:00</t>
+          <t>2026-10-02 10:45:20.519914+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>37152</t>
+          <t>37351</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>가상자산 활용 보이스피싱 피해 구제 확대 및 배달앱 원산지 표시 고지 의무화</t>
+          <t>법제처, 알기 쉬운 법령 만들기 20년을 돌아보고 미래를 이야기하다!</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157902&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157915&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -789,29 +789,29 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-01 10:15:19.890918+09:00</t>
+          <t>2026-10-01 15:15:21.104965+09:00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-01 10:15:19.890918+09:00</t>
+          <t>2026-10-01 15:15:21.104965+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>37151</t>
+          <t>37152</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Expanding Voice Phishing Damage Relief Utilizing Virtual Assets and ..</t>
+          <t>가상자산 활용 보이스피싱 피해 구제 확대 및 배달앱 원산지 표시 고지 의무화</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157904&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157902&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -843,17 +843,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>36341</t>
+          <t>37151</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>법제처, AI로 국민과 법의 거리를 좁힌다</t>
+          <t>Expanding Voice Phishing Damage Relief Utilizing Virtual Assets and ..</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157747&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157904&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -873,39 +873,39 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-09-29 10:30:21.085354+09:00</t>
+          <t>2026-10-01 10:15:19.890918+09:00</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-29 10:30:21.085354+09:00</t>
+          <t>2026-10-01 10:15:19.890918+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>33671</t>
+          <t>36341</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
+          <t>법제처, AI로 국민과 법의 거리를 좁힌다</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157747&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>법제조정법제관실</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -915,39 +915,39 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-09-22 15:30:19.394844+09:00</t>
+          <t>2026-09-29 10:30:21.085354+09:00</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-22 15:30:19.394844+09:00</t>
+          <t>2026-09-29 10:30:21.085354+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>33082</t>
+          <t>33671</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
+          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>법제조정법제관실</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -957,29 +957,29 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>31861</t>
+          <t>33082</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
+          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -999,39 +999,39 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>31651</t>
+          <t>31861</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
+          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>경제법제국</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1041,39 +1041,39 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>31201</t>
+          <t>31651</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
+          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>경제법제국</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1083,29 +1083,29 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>29141</t>
+          <t>31201</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
+          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1125,39 +1125,39 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>27851</t>
+          <t>29141</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
+          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1167,39 +1167,39 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>27461</t>
+          <t>27851</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>법제처, 제3회 특별성과 포상 수여</t>
+          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1209,39 +1209,39 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>25671</t>
+          <t>27461</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
+          <t>법제처, 제3회 특별성과 포상 수여</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1251,39 +1251,39 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>24842</t>
+          <t>25671</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
+          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1293,29 +1293,29 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>24841</t>
+          <t>24842</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
+          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1347,27 +1347,27 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>23411</t>
+          <t>24841</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
+          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1377,34 +1377,34 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>23231</t>
+          <t>23411</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
+          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>법제자문1담당관</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1419,39 +1419,39 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>14381</t>
+          <t>23231</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
+          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>법제자문1담당관</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1461,39 +1461,39 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>14121</t>
+          <t>14381</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>법제로 완성하는 국가대전환</t>
+          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1503,39 +1503,39 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>12952</t>
+          <t>14121</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
+          <t>법제로 완성하는 국가대전환</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1545,29 +1545,29 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>12951</t>
+          <t>12952</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
+          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1599,27 +1599,27 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>11761</t>
+          <t>12951</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
+          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>법제교육과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1629,34 +1629,34 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>11711</t>
+          <t>11761</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
+          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법제교육과</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1671,39 +1671,39 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>11311</t>
+          <t>11711</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>범정부 형벌 합리화 추진단 공식 출범</t>
+          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>파견</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1713,39 +1713,39 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>4471</t>
+          <t>11311</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
+          <t>범정부 형벌 합리화 추진단 공식 출범</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>파견</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1755,39 +1755,39 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1511</t>
+          <t>4471</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
+          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1797,39 +1797,39 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>491</t>
+          <t>1511</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
+          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1839,39 +1839,39 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>491</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
+          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1881,29 +1881,29 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
+          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1935,27 +1935,27 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
+          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1977,27 +1977,27 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
+          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2019,27 +2019,27 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
+          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2061,27 +2061,27 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
+          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2103,27 +2103,27 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
+          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2145,27 +2145,27 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
+          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2187,27 +2187,27 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2229,40 +2229,82 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>대변인실</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>자율주행 규제 합리화, 해외직구 안전 강화 등 국민보호 · 산업지원 새 법령 시행</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150819&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>대변인실</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="H45" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-10-29 15:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,22 +465,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>48631</t>
+          <t>48801</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>전통시장에서 찾는 일상 속 법 보물... K-법 생활발견 캠페인 ‘숨은 법 보물찾기’ 개최</t>
+          <t>법제처, 아동ㆍ청소년 대상 성범죄 예방을 위한 현장 간담회 개최</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=159333&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=159339&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법제조정법제관실</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -495,39 +495,39 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:15:19.676658+09:00</t>
+          <t>2026-10-29 14:30:18.950815+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:15:19.676658+09:00</t>
+          <t>2026-10-29 14:30:18.950815+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>47941</t>
+          <t>48631</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>실무경력 인정 범위를 넓혀, 청년의 사회진출 돕는다</t>
+          <t>전통시장에서 찾는 일상 속 법 보물... K-법 생활발견 캠페인 ‘숨은 법 보물찾기’ 개최</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=159220&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=159333&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>법령품질개선과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -537,39 +537,39 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-27 13:30:19.056395+09:00</t>
+          <t>2026-10-29 10:15:19.676658+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-27 13:30:19.056395+09:00</t>
+          <t>2026-10-29 10:15:19.676658+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>45631</t>
+          <t>47941</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>“법을 얼마나 알고 있나요?” 법제처, 청소년 골든벨 대회 개최</t>
+          <t>실무경력 인정 범위를 넓혀, 청년의 사회진출 돕는다</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158921&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=159220&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법령품질개선과</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -579,39 +579,39 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-21 17:15:20.296716+09:00</t>
+          <t>2026-10-27 13:30:19.056395+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-10-21 17:15:20.296716+09:00</t>
+          <t>2026-10-27 13:30:19.056395+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>45121</t>
+          <t>45631</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>국민의 생애주기에 맞춘 생활법령정보 서비스 발전 방안 논의</t>
+          <t>“법을 얼마나 알고 있나요?” 법제처, 청소년 골든벨 대회 개최</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158862&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158921&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -621,39 +621,39 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-20 14:45:19.906187+09:00</t>
+          <t>2026-10-21 17:15:20.296716+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-20 14:45:19.906187+09:00</t>
+          <t>2026-10-21 17:15:20.296716+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>41651</t>
+          <t>45121</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>법제처, 지방정부 등의 자치법규 입안을 위한 종합안내서 발간</t>
+          <t>국민의 생애주기에 맞춘 생활법령정보 서비스 발전 방안 논의</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158475&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158862&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -663,39 +663,39 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-12 10:00:18.987080+09:00</t>
+          <t>2026-10-20 14:45:19.906187+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-12 10:00:18.987080+09:00</t>
+          <t>2026-10-20 14:45:19.906187+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>37711</t>
+          <t>41651</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>“행정기본법 제정 5주년, 새로운 길을 찾다”</t>
+          <t>법제처, 지방정부 등의 자치법규 입안을 위한 종합안내서 발간</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157976&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158475&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -705,34 +705,34 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-02 14:00:20.071730+09:00</t>
+          <t>2026-10-12 10:00:18.987080+09:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-02 14:00:20.071730+09:00</t>
+          <t>2026-10-12 10:00:18.987080+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>37581</t>
+          <t>37711</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>국민이 직접 뽑은 ‘대표 알기 쉬운 법령 용어’에 “사위(詐僞) → 거짓/속임수” 등 5개 선정</t>
+          <t>“행정기본법 제정 5주년, 새로운 길을 찾다”</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157972&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157976&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -747,29 +747,29 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-02 10:45:20.519914+09:00</t>
+          <t>2026-10-02 14:00:20.071730+09:00</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-02 10:45:20.519914+09:00</t>
+          <t>2026-10-02 14:00:20.071730+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>37351</t>
+          <t>37581</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>법제처, 알기 쉬운 법령 만들기 20년을 돌아보고 미래를 이야기하다!</t>
+          <t>국민이 직접 뽑은 ‘대표 알기 쉬운 법령 용어’에 “사위(詐僞) → 거짓/속임수” 등 5개 선정</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157915&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157972&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -789,34 +789,34 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-01 15:15:21.104965+09:00</t>
+          <t>2026-10-02 10:45:20.519914+09:00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-01 15:15:21.104965+09:00</t>
+          <t>2026-10-02 10:45:20.519914+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>37152</t>
+          <t>37351</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>가상자산 활용 보이스피싱 피해 구제 확대 및 배달앱 원산지 표시 고지 의무화</t>
+          <t>법제처, 알기 쉬운 법령 만들기 20년을 돌아보고 미래를 이야기하다!</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157902&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157915&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -831,29 +831,29 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-01 10:15:19.890918+09:00</t>
+          <t>2026-10-01 15:15:21.104965+09:00</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-01 10:15:19.890918+09:00</t>
+          <t>2026-10-01 15:15:21.104965+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>37151</t>
+          <t>37152</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Expanding Voice Phishing Damage Relief Utilizing Virtual Assets and ..</t>
+          <t>가상자산 활용 보이스피싱 피해 구제 확대 및 배달앱 원산지 표시 고지 의무화</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157904&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157902&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -885,17 +885,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>36341</t>
+          <t>37151</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>법제처, AI로 국민과 법의 거리를 좁힌다</t>
+          <t>Expanding Voice Phishing Damage Relief Utilizing Virtual Assets and ..</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157747&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157904&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -905,7 +905,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -915,39 +915,39 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-09-29 10:30:21.085354+09:00</t>
+          <t>2026-10-01 10:15:19.890918+09:00</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-29 10:30:21.085354+09:00</t>
+          <t>2026-10-01 10:15:19.890918+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>33671</t>
+          <t>36341</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
+          <t>법제처, AI로 국민과 법의 거리를 좁힌다</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157747&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>법제조정법제관실</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -957,39 +957,39 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-09-22 15:30:19.394844+09:00</t>
+          <t>2026-09-29 10:30:21.085354+09:00</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-22 15:30:19.394844+09:00</t>
+          <t>2026-09-29 10:30:21.085354+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>33082</t>
+          <t>33671</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
+          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>법제조정법제관실</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -999,29 +999,29 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>31861</t>
+          <t>33082</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
+          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1041,39 +1041,39 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>31651</t>
+          <t>31861</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
+          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>경제법제국</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1083,39 +1083,39 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>31201</t>
+          <t>31651</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
+          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>경제법제국</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1125,29 +1125,29 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>29141</t>
+          <t>31201</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
+          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1157,7 +1157,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1167,39 +1167,39 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>27851</t>
+          <t>29141</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
+          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1209,39 +1209,39 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>27461</t>
+          <t>27851</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>법제처, 제3회 특별성과 포상 수여</t>
+          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1251,39 +1251,39 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>25671</t>
+          <t>27461</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
+          <t>법제처, 제3회 특별성과 포상 수여</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1293,39 +1293,39 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>24842</t>
+          <t>25671</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
+          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1335,29 +1335,29 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>24841</t>
+          <t>24842</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
+          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1389,27 +1389,27 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>23411</t>
+          <t>24841</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
+          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1419,34 +1419,34 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>23231</t>
+          <t>23411</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
+          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>법제자문1담당관</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1461,39 +1461,39 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>14381</t>
+          <t>23231</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
+          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>법제자문1담당관</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1503,39 +1503,39 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>14121</t>
+          <t>14381</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>법제로 완성하는 국가대전환</t>
+          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1545,39 +1545,39 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>12952</t>
+          <t>14121</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
+          <t>법제로 완성하는 국가대전환</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1587,29 +1587,29 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>12951</t>
+          <t>12952</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
+          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1641,27 +1641,27 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>11761</t>
+          <t>12951</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
+          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>법제교육과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1671,34 +1671,34 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>11711</t>
+          <t>11761</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
+          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법제교육과</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1713,39 +1713,39 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>11311</t>
+          <t>11711</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>범정부 형벌 합리화 추진단 공식 출범</t>
+          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>파견</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1755,39 +1755,39 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>4471</t>
+          <t>11311</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
+          <t>범정부 형벌 합리화 추진단 공식 출범</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>파견</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1797,39 +1797,39 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1511</t>
+          <t>4471</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
+          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1839,39 +1839,39 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>491</t>
+          <t>1511</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
+          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1881,39 +1881,39 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>491</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
+          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1923,29 +1923,29 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
+          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1977,27 +1977,27 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
+          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2019,27 +2019,27 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
+          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2061,27 +2061,27 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
+          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2103,27 +2103,27 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
+          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2145,27 +2145,27 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
+          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2187,27 +2187,27 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
+          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2229,27 +2229,27 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2271,40 +2271,82 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>대변인실</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>자율주행 규제 합리화, 해외직구 안전 강화 등 국민보호 · 산업지원 새 법령 시행</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150819&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>대변인실</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="H46" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-10-30 11:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/all.xlsx
+++ b/docs/snapshot/downloads/all.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,27 +465,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>48801</t>
+          <t>49051</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>법제처, 아동ㆍ청소년 대상 성범죄 예방을 위한 현장 간담회 개최</t>
+          <t>문화ㆍ관광ㆍ산업 등 분야 어려운 법령, 한눈에 이해되는 시각 콘텐츠로 본다</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=159339&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=159415&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>법제조정법제관실</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -495,34 +495,34 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:30:18.950815+09:00</t>
+          <t>2026-10-30 10:30:19.059936+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:30:18.950815+09:00</t>
+          <t>2026-10-30 10:30:19.059936+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>48631</t>
+          <t>48801</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>전통시장에서 찾는 일상 속 법 보물... K-법 생활발견 캠페인 ‘숨은 법 보물찾기’ 개최</t>
+          <t>법제처, 아동ㆍ청소년 대상 성범죄 예방을 위한 현장 간담회 개최</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=159333&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=159339&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법제조정법제관실</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -537,39 +537,39 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-29 10:15:19.676658+09:00</t>
+          <t>2026-10-29 14:30:18.950815+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-29 10:15:19.676658+09:00</t>
+          <t>2026-10-29 14:30:18.950815+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>47941</t>
+          <t>48631</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>실무경력 인정 범위를 넓혀, 청년의 사회진출 돕는다</t>
+          <t>전통시장에서 찾는 일상 속 법 보물... K-법 생활발견 캠페인 ‘숨은 법 보물찾기’ 개최</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=159220&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=159333&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>법령품질개선과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -579,39 +579,39 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-27 13:30:19.056395+09:00</t>
+          <t>2026-10-29 10:15:19.676658+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-10-27 13:30:19.056395+09:00</t>
+          <t>2026-10-29 10:15:19.676658+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>45631</t>
+          <t>47941</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>“법을 얼마나 알고 있나요?” 법제처, 청소년 골든벨 대회 개최</t>
+          <t>실무경력 인정 범위를 넓혀, 청년의 사회진출 돕는다</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158921&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=159220&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법령품질개선과</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -621,39 +621,39 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-21 17:15:20.296716+09:00</t>
+          <t>2026-10-27 13:30:19.056395+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-21 17:15:20.296716+09:00</t>
+          <t>2026-10-27 13:30:19.056395+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>45121</t>
+          <t>45631</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>국민의 생애주기에 맞춘 생활법령정보 서비스 발전 방안 논의</t>
+          <t>“법을 얼마나 알고 있나요?” 법제처, 청소년 골든벨 대회 개최</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158862&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158921&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -663,39 +663,39 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-20 14:45:19.906187+09:00</t>
+          <t>2026-10-21 17:15:20.296716+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-20 14:45:19.906187+09:00</t>
+          <t>2026-10-21 17:15:20.296716+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>41651</t>
+          <t>45121</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>법제처, 지방정부 등의 자치법규 입안을 위한 종합안내서 발간</t>
+          <t>국민의 생애주기에 맞춘 생활법령정보 서비스 발전 방안 논의</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158475&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158862&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -705,39 +705,39 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-12 10:00:18.987080+09:00</t>
+          <t>2026-10-20 14:45:19.906187+09:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-12 10:00:18.987080+09:00</t>
+          <t>2026-10-20 14:45:19.906187+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>37711</t>
+          <t>41651</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>“행정기본법 제정 5주년, 새로운 길을 찾다”</t>
+          <t>법제처, 지방정부 등의 자치법규 입안을 위한 종합안내서 발간</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157976&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=158475&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -747,34 +747,34 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-10-02 14:00:20.071730+09:00</t>
+          <t>2026-10-12 10:00:18.987080+09:00</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-02 14:00:20.071730+09:00</t>
+          <t>2026-10-12 10:00:18.987080+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>37581</t>
+          <t>37711</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>국민이 직접 뽑은 ‘대표 알기 쉬운 법령 용어’에 “사위(詐僞) → 거짓/속임수” 등 5개 선정</t>
+          <t>“행정기본법 제정 5주년, 새로운 길을 찾다”</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157972&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157976&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -789,29 +789,29 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-10-02 10:45:20.519914+09:00</t>
+          <t>2026-10-02 14:00:20.071730+09:00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-02 10:45:20.519914+09:00</t>
+          <t>2026-10-02 14:00:20.071730+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>37351</t>
+          <t>37581</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>법제처, 알기 쉬운 법령 만들기 20년을 돌아보고 미래를 이야기하다!</t>
+          <t>국민이 직접 뽑은 ‘대표 알기 쉬운 법령 용어’에 “사위(詐僞) → 거짓/속임수” 등 5개 선정</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157915&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157972&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -831,34 +831,34 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-10-01 15:15:21.104965+09:00</t>
+          <t>2026-10-02 10:45:20.519914+09:00</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-01 15:15:21.104965+09:00</t>
+          <t>2026-10-02 10:45:20.519914+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>37152</t>
+          <t>37351</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>가상자산 활용 보이스피싱 피해 구제 확대 및 배달앱 원산지 표시 고지 의무화</t>
+          <t>법제처, 알기 쉬운 법령 만들기 20년을 돌아보고 미래를 이야기하다!</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157902&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157915&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -873,29 +873,29 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-10-01 10:15:19.890918+09:00</t>
+          <t>2026-10-01 15:15:21.104965+09:00</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-01 10:15:19.890918+09:00</t>
+          <t>2026-10-01 15:15:21.104965+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>37151</t>
+          <t>37152</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Expanding Voice Phishing Damage Relief Utilizing Virtual Assets and ..</t>
+          <t>가상자산 활용 보이스피싱 피해 구제 확대 및 배달앱 원산지 표시 고지 의무화</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157904&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157902&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -927,17 +927,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>36341</t>
+          <t>37151</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>법제처, AI로 국민과 법의 거리를 좁힌다</t>
+          <t>Expanding Voice Phishing Damage Relief Utilizing Virtual Assets and ..</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157747&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157904&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -957,39 +957,39 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-09-29 10:30:21.085354+09:00</t>
+          <t>2026-10-01 10:15:19.890918+09:00</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-29 10:30:21.085354+09:00</t>
+          <t>2026-10-01 10:15:19.890918+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>33671</t>
+          <t>36341</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
+          <t>법제처, AI로 국민과 법의 거리를 좁힌다</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157747&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>법제조정법제관실</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -999,39 +999,39 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-09-22 15:30:19.394844+09:00</t>
+          <t>2026-09-29 10:30:21.085354+09:00</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-22 15:30:19.394844+09:00</t>
+          <t>2026-09-29 10:30:21.085354+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>33082</t>
+          <t>33671</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
+          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>법제조정법제관실</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1041,29 +1041,29 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>31861</t>
+          <t>33082</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
+          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1083,39 +1083,39 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>31651</t>
+          <t>31861</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
+          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>경제법제국</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1125,39 +1125,39 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>31201</t>
+          <t>31651</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
+          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>경제법제국</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1167,29 +1167,29 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>29141</t>
+          <t>31201</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
+          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1199,7 +1199,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1209,39 +1209,39 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>27851</t>
+          <t>29141</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
+          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1251,39 +1251,39 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>27461</t>
+          <t>27851</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>법제처, 제3회 특별성과 포상 수여</t>
+          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1293,39 +1293,39 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>25671</t>
+          <t>27461</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
+          <t>법제처, 제3회 특별성과 포상 수여</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1335,39 +1335,39 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>24842</t>
+          <t>25671</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
+          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1377,29 +1377,29 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>24841</t>
+          <t>24842</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
+          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1431,27 +1431,27 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>23411</t>
+          <t>24841</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
+          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1461,34 +1461,34 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>23231</t>
+          <t>23411</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
+          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>법제자문1담당관</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1503,39 +1503,39 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>14381</t>
+          <t>23231</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
+          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>법제자문1담당관</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1545,39 +1545,39 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>14121</t>
+          <t>14381</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>법제로 완성하는 국가대전환</t>
+          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1587,39 +1587,39 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>12952</t>
+          <t>14121</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
+          <t>법제로 완성하는 국가대전환</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1629,29 +1629,29 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>12951</t>
+          <t>12952</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
+          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1683,27 +1683,27 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>11761</t>
+          <t>12951</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
+          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>법제교육과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1713,34 +1713,34 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>11711</t>
+          <t>11761</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
+          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법제교육과</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1755,39 +1755,39 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>11311</t>
+          <t>11711</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>범정부 형벌 합리화 추진단 공식 출범</t>
+          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>파견</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1797,39 +1797,39 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>4471</t>
+          <t>11311</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
+          <t>범정부 형벌 합리화 추진단 공식 출범</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>파견</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1839,39 +1839,39 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1511</t>
+          <t>4471</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
+          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1881,39 +1881,39 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>491</t>
+          <t>1511</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
+          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1923,39 +1923,39 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>491</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
+          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1965,29 +1965,29 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
+          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2019,27 +2019,27 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
+          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2061,27 +2061,27 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
+          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2103,27 +2103,27 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
+          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2145,27 +2145,27 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
+          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2187,27 +2187,27 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
+          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2229,27 +2229,27 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
+          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2271,27 +2271,27 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2313,40 +2313,82 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>대변인실</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>자율주행 규제 합리화, 해외직구 안전 강화 등 국민보호 · 산업지원 새 법령 시행</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150819&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>대변인실</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="H47" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>

</xml_diff>